<commit_message>
3.1.0 Se agregan nombres a los tickets
</commit_message>
<xml_diff>
--- a/static/plantillas/XXX-XXX-XXX-X-XXX-XXX-XXX DictamenPruebas PRUEBAS.xlsx
+++ b/static/plantillas/XXX-XXX-XXX-X-XXX-XXX-XXX DictamenPruebas PRUEBAS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BID-eduardo.hernande\Desktop\extractor\excel_extractor\static\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{677195DC-77B5-4E43-B534-F8F8008C02F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7840C64D-7120-46E7-A839-42C5B12D70F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{1A5253DA-6AA8-4BED-9DA7-B3D404B25E3E}"/>
   </bookViews>
@@ -818,7 +818,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="95">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1045,38 +1045,41 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1096,10 +1099,65 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>361650</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>558235</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagen 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{74F77198-92E4-41C3-A36A-E8C924810A17}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4476750" y="5168900"/>
+          <a:ext cx="742650" cy="431235"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1137,7 +1195,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1243,7 +1301,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1385,7 +1443,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1394,7 +1452,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9D327AB-10D1-4242-8DFB-6C38C435BDAB}">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="16" style="1" customWidth="1"/>
     <col min="2" max="2" width="32.26953125" style="1" customWidth="1"/>
@@ -1488,7 +1546,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A99367A2-59BD-4B7E-A698-13023E16A06B}">
   <dimension ref="A2:Q37"/>
-  <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="11.453125" style="1" customWidth="1"/>
     <col min="2" max="2" width="16.7265625" style="1" customWidth="1"/>
@@ -1578,42 +1636,42 @@
       <c r="P3" s="45"/>
       <c r="Q3" s="45"/>
     </row>
-    <row r="5" spans="1:17">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:17" ht="14" customHeight="1">
+      <c r="A5" s="84" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="84" t="s">
+      <c r="B5" s="87" t="s">
         <v>54</v>
       </c>
-      <c r="C5" s="84"/>
-      <c r="D5" s="84"/>
-      <c r="E5" s="90" t="s">
+      <c r="C5" s="87"/>
+      <c r="D5" s="87"/>
+      <c r="E5" s="91" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="90"/>
-      <c r="G5" s="90"/>
-      <c r="H5" s="90"/>
-      <c r="I5" s="90"/>
-      <c r="J5" s="91"/>
-      <c r="K5" s="92" t="s">
+      <c r="F5" s="91"/>
+      <c r="G5" s="91"/>
+      <c r="H5" s="91"/>
+      <c r="I5" s="91"/>
+      <c r="J5" s="92"/>
+      <c r="K5" s="93" t="s">
         <v>58</v>
       </c>
-      <c r="L5" s="93"/>
-      <c r="M5" s="93"/>
-      <c r="N5" s="93"/>
-      <c r="O5" s="93"/>
-      <c r="P5" s="93"/>
-      <c r="Q5" s="94"/>
-    </row>
-    <row r="6" spans="1:17">
-      <c r="A6" s="2" t="s">
+      <c r="L5" s="94"/>
+      <c r="M5" s="94"/>
+      <c r="N5" s="94"/>
+      <c r="O5" s="94"/>
+      <c r="P5" s="94"/>
+      <c r="Q5" s="95"/>
+    </row>
+    <row r="6" spans="1:17" ht="18" customHeight="1">
+      <c r="A6" s="84" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="84" t="s">
+      <c r="B6" s="87" t="s">
         <v>55</v>
       </c>
-      <c r="C6" s="84"/>
-      <c r="D6" s="84"/>
+      <c r="C6" s="87"/>
+      <c r="D6" s="87"/>
       <c r="E6" s="85" t="s">
         <v>7</v>
       </c>
@@ -1622,15 +1680,15 @@
       <c r="H6" s="85"/>
       <c r="I6" s="85"/>
       <c r="J6" s="86"/>
-      <c r="K6" s="87" t="s">
+      <c r="K6" s="88" t="s">
         <v>59</v>
       </c>
-      <c r="L6" s="88"/>
-      <c r="M6" s="88"/>
-      <c r="N6" s="88"/>
-      <c r="O6" s="88"/>
-      <c r="P6" s="88"/>
-      <c r="Q6" s="89"/>
+      <c r="L6" s="89"/>
+      <c r="M6" s="89"/>
+      <c r="N6" s="89"/>
+      <c r="O6" s="89"/>
+      <c r="P6" s="89"/>
+      <c r="Q6" s="90"/>
     </row>
     <row r="7" spans="1:17">
       <c r="A7" s="3" t="s">
@@ -2184,6 +2242,7 @@
 Versión: 02 
 Emisión: 25-04-25</oddHeader>
   </headerFooter>
-  <legacyDrawingHF r:id="rId2"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawingHF r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
3.1.4 Se modifica la plantilla del dictamen
</commit_message>
<xml_diff>
--- a/static/plantillas/XXX-XXX-XXX-X-XXX-XXX-XXX DictamenPruebas PRUEBAS.xlsx
+++ b/static/plantillas/XXX-XXX-XXX-X-XXX-XXX-XXX DictamenPruebas PRUEBAS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BID-eduardo.hernande\Desktop\extractor\excel_extractor\static\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7840C64D-7120-46E7-A839-42C5B12D70F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA030A52-C14E-4AA9-A931-02201BB29B8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{1A5253DA-6AA8-4BED-9DA7-B3D404B25E3E}"/>
   </bookViews>
@@ -818,7 +818,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -897,6 +897,9 @@
     <xf numFmtId="49" fontId="5" fillId="2" borderId="2" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1045,8 +1048,8 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1054,9 +1057,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1064,6 +1064,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1569,12 +1572,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" ht="28.5" customHeight="1">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="35"/>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
       <c r="E2" s="17" t="s">
         <v>1</v>
       </c>
@@ -1616,70 +1619,70 @@
       </c>
     </row>
     <row r="3" spans="1:17">
-      <c r="A3" s="45" t="s">
+      <c r="A3" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="45"/>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="45"/>
-      <c r="F3" s="45"/>
-      <c r="G3" s="45"/>
-      <c r="H3" s="45"/>
-      <c r="I3" s="45"/>
-      <c r="J3" s="45"/>
-      <c r="K3" s="45"/>
-      <c r="L3" s="45"/>
-      <c r="M3" s="45"/>
-      <c r="N3" s="45"/>
-      <c r="O3" s="45"/>
-      <c r="P3" s="45"/>
-      <c r="Q3" s="45"/>
+      <c r="B3" s="46"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="46"/>
+      <c r="G3" s="46"/>
+      <c r="H3" s="46"/>
+      <c r="I3" s="46"/>
+      <c r="J3" s="46"/>
+      <c r="K3" s="46"/>
+      <c r="L3" s="46"/>
+      <c r="M3" s="46"/>
+      <c r="N3" s="46"/>
+      <c r="O3" s="46"/>
+      <c r="P3" s="46"/>
+      <c r="Q3" s="46"/>
     </row>
     <row r="5" spans="1:17" ht="14" customHeight="1">
-      <c r="A5" s="84" t="s">
+      <c r="A5" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="87" t="s">
+      <c r="B5" s="91" t="s">
         <v>54</v>
       </c>
-      <c r="C5" s="87"/>
-      <c r="D5" s="87"/>
-      <c r="E5" s="91" t="s">
+      <c r="C5" s="91"/>
+      <c r="D5" s="91"/>
+      <c r="E5" s="92" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="91"/>
-      <c r="G5" s="91"/>
-      <c r="H5" s="91"/>
-      <c r="I5" s="91"/>
-      <c r="J5" s="92"/>
-      <c r="K5" s="93" t="s">
+      <c r="F5" s="92"/>
+      <c r="G5" s="92"/>
+      <c r="H5" s="92"/>
+      <c r="I5" s="92"/>
+      <c r="J5" s="93"/>
+      <c r="K5" s="94" t="s">
         <v>58</v>
       </c>
-      <c r="L5" s="94"/>
-      <c r="M5" s="94"/>
-      <c r="N5" s="94"/>
-      <c r="O5" s="94"/>
-      <c r="P5" s="94"/>
-      <c r="Q5" s="95"/>
+      <c r="L5" s="95"/>
+      <c r="M5" s="95"/>
+      <c r="N5" s="95"/>
+      <c r="O5" s="95"/>
+      <c r="P5" s="95"/>
+      <c r="Q5" s="96"/>
     </row>
     <row r="6" spans="1:17" ht="18" customHeight="1">
-      <c r="A6" s="84" t="s">
+      <c r="A6" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="87" t="s">
+      <c r="B6" s="85" t="s">
         <v>55</v>
       </c>
-      <c r="C6" s="87"/>
-      <c r="D6" s="87"/>
-      <c r="E6" s="85" t="s">
+      <c r="C6" s="85"/>
+      <c r="D6" s="85"/>
+      <c r="E6" s="86" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="85"/>
-      <c r="G6" s="85"/>
-      <c r="H6" s="85"/>
-      <c r="I6" s="85"/>
-      <c r="J6" s="86"/>
+      <c r="F6" s="86"/>
+      <c r="G6" s="86"/>
+      <c r="H6" s="86"/>
+      <c r="I6" s="86"/>
+      <c r="J6" s="87"/>
       <c r="K6" s="88" t="s">
         <v>59</v>
       </c>
@@ -1705,18 +1708,18 @@
       <c r="H7" s="7"/>
       <c r="I7" s="7"/>
       <c r="J7" s="8"/>
-      <c r="K7" s="72" t="s">
+      <c r="K7" s="73" t="s">
         <v>9</v>
       </c>
-      <c r="L7" s="73"/>
-      <c r="M7" s="57" t="s">
+      <c r="L7" s="74"/>
+      <c r="M7" s="58" t="s">
         <v>44</v>
       </c>
-      <c r="N7" s="59"/>
-      <c r="O7" s="72" t="s">
+      <c r="N7" s="60"/>
+      <c r="O7" s="73" t="s">
         <v>10</v>
       </c>
-      <c r="P7" s="73"/>
+      <c r="P7" s="74"/>
       <c r="Q7" s="9" t="s">
         <v>44</v>
       </c>
@@ -1725,124 +1728,124 @@
       <c r="A8" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="74" t="s">
+      <c r="B8" s="75" t="s">
         <v>45</v>
       </c>
-      <c r="C8" s="74"/>
-      <c r="D8" s="74"/>
-      <c r="E8" s="74"/>
-      <c r="F8" s="74"/>
-      <c r="G8" s="74"/>
-      <c r="H8" s="74"/>
-      <c r="I8" s="74"/>
-      <c r="J8" s="74"/>
-      <c r="K8" s="74"/>
-      <c r="L8" s="74"/>
-      <c r="M8" s="74"/>
-      <c r="N8" s="74"/>
-      <c r="O8" s="74"/>
-      <c r="P8" s="74"/>
-      <c r="Q8" s="74"/>
+      <c r="C8" s="75"/>
+      <c r="D8" s="75"/>
+      <c r="E8" s="75"/>
+      <c r="F8" s="75"/>
+      <c r="G8" s="75"/>
+      <c r="H8" s="75"/>
+      <c r="I8" s="75"/>
+      <c r="J8" s="75"/>
+      <c r="K8" s="75"/>
+      <c r="L8" s="75"/>
+      <c r="M8" s="75"/>
+      <c r="N8" s="75"/>
+      <c r="O8" s="75"/>
+      <c r="P8" s="75"/>
+      <c r="Q8" s="75"/>
     </row>
     <row r="9" spans="1:17">
-      <c r="A9" s="70" t="s">
+      <c r="A9" s="71" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="75"/>
-      <c r="C9" s="76" t="s">
+      <c r="B9" s="76"/>
+      <c r="C9" s="77" t="s">
         <v>45</v>
       </c>
-      <c r="D9" s="76"/>
-      <c r="E9" s="76"/>
-      <c r="F9" s="76"/>
-      <c r="G9" s="76"/>
-      <c r="H9" s="76"/>
-      <c r="I9" s="76"/>
-      <c r="J9" s="76"/>
-      <c r="K9" s="76"/>
-      <c r="L9" s="76"/>
-      <c r="M9" s="76"/>
-      <c r="N9" s="76"/>
-      <c r="O9" s="76"/>
-      <c r="P9" s="76"/>
-      <c r="Q9" s="77"/>
+      <c r="D9" s="77"/>
+      <c r="E9" s="77"/>
+      <c r="F9" s="77"/>
+      <c r="G9" s="77"/>
+      <c r="H9" s="77"/>
+      <c r="I9" s="77"/>
+      <c r="J9" s="77"/>
+      <c r="K9" s="77"/>
+      <c r="L9" s="77"/>
+      <c r="M9" s="77"/>
+      <c r="N9" s="77"/>
+      <c r="O9" s="77"/>
+      <c r="P9" s="77"/>
+      <c r="Q9" s="78"/>
     </row>
     <row r="10" spans="1:17">
-      <c r="A10" s="78" t="s">
+      <c r="A10" s="79" t="s">
         <v>13</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="79" t="s">
+      <c r="C10" s="80" t="s">
         <v>44</v>
       </c>
-      <c r="D10" s="79"/>
-      <c r="E10" s="79"/>
-      <c r="F10" s="79"/>
-      <c r="G10" s="79"/>
-      <c r="H10" s="79"/>
-      <c r="I10" s="79"/>
-      <c r="J10" s="79"/>
-      <c r="K10" s="79"/>
-      <c r="L10" s="79"/>
-      <c r="M10" s="79"/>
-      <c r="N10" s="79"/>
-      <c r="O10" s="79"/>
-      <c r="P10" s="79"/>
-      <c r="Q10" s="79"/>
+      <c r="D10" s="80"/>
+      <c r="E10" s="80"/>
+      <c r="F10" s="80"/>
+      <c r="G10" s="80"/>
+      <c r="H10" s="80"/>
+      <c r="I10" s="80"/>
+      <c r="J10" s="80"/>
+      <c r="K10" s="80"/>
+      <c r="L10" s="80"/>
+      <c r="M10" s="80"/>
+      <c r="N10" s="80"/>
+      <c r="O10" s="80"/>
+      <c r="P10" s="80"/>
+      <c r="Q10" s="80"/>
     </row>
     <row r="11" spans="1:17">
-      <c r="A11" s="78"/>
+      <c r="A11" s="79"/>
       <c r="B11" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="79" t="s">
+      <c r="C11" s="80" t="s">
         <v>44</v>
       </c>
-      <c r="D11" s="79"/>
-      <c r="E11" s="79"/>
-      <c r="F11" s="79"/>
-      <c r="G11" s="79"/>
-      <c r="H11" s="79"/>
-      <c r="I11" s="79"/>
-      <c r="J11" s="79"/>
-      <c r="K11" s="79"/>
-      <c r="L11" s="79"/>
-      <c r="M11" s="79"/>
-      <c r="N11" s="79"/>
-      <c r="O11" s="79"/>
-      <c r="P11" s="79"/>
-      <c r="Q11" s="79"/>
+      <c r="D11" s="80"/>
+      <c r="E11" s="80"/>
+      <c r="F11" s="80"/>
+      <c r="G11" s="80"/>
+      <c r="H11" s="80"/>
+      <c r="I11" s="80"/>
+      <c r="J11" s="80"/>
+      <c r="K11" s="80"/>
+      <c r="L11" s="80"/>
+      <c r="M11" s="80"/>
+      <c r="N11" s="80"/>
+      <c r="O11" s="80"/>
+      <c r="P11" s="80"/>
+      <c r="Q11" s="80"/>
     </row>
     <row r="12" spans="1:17">
       <c r="A12" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="80" t="s">
+      <c r="B12" s="81" t="s">
         <v>44</v>
       </c>
-      <c r="C12" s="81"/>
-      <c r="D12" s="81"/>
-      <c r="E12" s="81"/>
-      <c r="F12" s="81"/>
-      <c r="G12" s="81"/>
-      <c r="H12" s="81"/>
-      <c r="I12" s="81"/>
-      <c r="J12" s="81"/>
-      <c r="K12" s="81"/>
-      <c r="L12" s="81"/>
-      <c r="M12" s="81"/>
-      <c r="N12" s="81"/>
-      <c r="O12" s="81"/>
-      <c r="P12" s="81"/>
-      <c r="Q12" s="82"/>
+      <c r="C12" s="82"/>
+      <c r="D12" s="82"/>
+      <c r="E12" s="82"/>
+      <c r="F12" s="82"/>
+      <c r="G12" s="82"/>
+      <c r="H12" s="82"/>
+      <c r="I12" s="82"/>
+      <c r="J12" s="82"/>
+      <c r="K12" s="82"/>
+      <c r="L12" s="82"/>
+      <c r="M12" s="82"/>
+      <c r="N12" s="82"/>
+      <c r="O12" s="82"/>
+      <c r="P12" s="82"/>
+      <c r="Q12" s="83"/>
     </row>
     <row r="13" spans="1:17">
-      <c r="A13" s="70" t="s">
+      <c r="A13" s="71" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="83"/>
+      <c r="B13" s="84"/>
       <c r="C13" s="12" t="s">
         <v>44</v>
       </c>
@@ -1862,10 +1865,10 @@
       <c r="Q13" s="14"/>
     </row>
     <row r="14" spans="1:17">
-      <c r="A14" s="70" t="s">
+      <c r="A14" s="71" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="71"/>
+      <c r="B14" s="72"/>
       <c r="C14" s="15" t="s">
         <v>44</v>
       </c>
@@ -1888,296 +1891,298 @@
       <c r="A15" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="41" t="s">
+      <c r="B15" s="42" t="s">
         <v>44</v>
       </c>
-      <c r="C15" s="41"/>
-      <c r="D15" s="41"/>
-      <c r="E15" s="41"/>
-      <c r="F15" s="41"/>
-      <c r="G15" s="41"/>
-      <c r="H15" s="41"/>
-      <c r="I15" s="41"/>
-      <c r="J15" s="41"/>
-      <c r="K15" s="41"/>
-      <c r="L15" s="41"/>
-      <c r="M15" s="41"/>
-      <c r="N15" s="41"/>
-      <c r="O15" s="41"/>
-      <c r="P15" s="41"/>
-      <c r="Q15" s="41"/>
+      <c r="C15" s="42"/>
+      <c r="D15" s="42"/>
+      <c r="E15" s="42"/>
+      <c r="F15" s="42"/>
+      <c r="G15" s="42"/>
+      <c r="H15" s="42"/>
+      <c r="I15" s="42"/>
+      <c r="J15" s="42"/>
+      <c r="K15" s="42"/>
+      <c r="L15" s="42"/>
+      <c r="M15" s="42"/>
+      <c r="N15" s="42"/>
+      <c r="O15" s="42"/>
+      <c r="P15" s="42"/>
+      <c r="Q15" s="42"/>
     </row>
     <row r="16" spans="1:17">
-      <c r="A16" s="43" t="s">
+      <c r="A16" s="44" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="54"/>
-      <c r="C16" s="55"/>
-      <c r="D16" s="55"/>
-      <c r="E16" s="55"/>
-      <c r="F16" s="55"/>
-      <c r="G16" s="54"/>
-      <c r="H16" s="54"/>
-      <c r="I16" s="54"/>
-      <c r="J16" s="54"/>
-      <c r="K16" s="54"/>
-      <c r="L16" s="54"/>
-      <c r="M16" s="55"/>
-      <c r="N16" s="55"/>
-      <c r="O16" s="55"/>
-      <c r="P16" s="55"/>
-      <c r="Q16" s="56"/>
+      <c r="B16" s="55"/>
+      <c r="C16" s="56"/>
+      <c r="D16" s="56"/>
+      <c r="E16" s="56"/>
+      <c r="F16" s="56"/>
+      <c r="G16" s="55"/>
+      <c r="H16" s="55"/>
+      <c r="I16" s="55"/>
+      <c r="J16" s="55"/>
+      <c r="K16" s="55"/>
+      <c r="L16" s="55"/>
+      <c r="M16" s="56"/>
+      <c r="N16" s="56"/>
+      <c r="O16" s="56"/>
+      <c r="P16" s="56"/>
+      <c r="Q16" s="57"/>
     </row>
     <row r="17" spans="1:17">
-      <c r="A17" s="47" t="s">
+      <c r="A17" s="48" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="47"/>
-      <c r="C17" s="57"/>
-      <c r="D17" s="58"/>
-      <c r="E17" s="58"/>
-      <c r="F17" s="59"/>
-      <c r="G17" s="60" t="s">
+      <c r="B17" s="48"/>
+      <c r="C17" s="58"/>
+      <c r="D17" s="59"/>
+      <c r="E17" s="59"/>
+      <c r="F17" s="60"/>
+      <c r="G17" s="61" t="s">
         <v>22</v>
       </c>
-      <c r="H17" s="61"/>
-      <c r="I17" s="61"/>
-      <c r="J17" s="61"/>
-      <c r="K17" s="61"/>
-      <c r="L17" s="62"/>
-      <c r="M17" s="63">
+      <c r="H17" s="62"/>
+      <c r="I17" s="62"/>
+      <c r="J17" s="62"/>
+      <c r="K17" s="62"/>
+      <c r="L17" s="63"/>
+      <c r="M17" s="64">
         <v>16</v>
       </c>
-      <c r="N17" s="64"/>
-      <c r="O17" s="65" t="s">
+      <c r="N17" s="65"/>
+      <c r="O17" s="66" t="s">
         <v>23</v>
       </c>
-      <c r="P17" s="65"/>
-      <c r="Q17" s="66"/>
+      <c r="P17" s="66"/>
+      <c r="Q17" s="67"/>
     </row>
     <row r="18" spans="1:17">
-      <c r="A18" s="39" t="s">
+      <c r="A18" s="40" t="s">
         <v>24</v>
       </c>
-      <c r="B18" s="40"/>
-      <c r="C18" s="41">
+      <c r="B18" s="41"/>
+      <c r="C18" s="42">
         <v>1</v>
       </c>
-      <c r="D18" s="41"/>
-      <c r="E18" s="41"/>
-      <c r="F18" s="42"/>
-      <c r="G18" s="43" t="s">
+      <c r="D18" s="42"/>
+      <c r="E18" s="42"/>
+      <c r="F18" s="43"/>
+      <c r="G18" s="44" t="s">
         <v>25</v>
       </c>
-      <c r="H18" s="43"/>
-      <c r="I18" s="43"/>
-      <c r="J18" s="43"/>
-      <c r="K18" s="43"/>
-      <c r="L18" s="43"/>
-      <c r="M18" s="44">
+      <c r="H18" s="44"/>
+      <c r="I18" s="44"/>
+      <c r="J18" s="44"/>
+      <c r="K18" s="44"/>
+      <c r="L18" s="44"/>
+      <c r="M18" s="45">
         <v>16</v>
       </c>
-      <c r="N18" s="44"/>
-      <c r="O18" s="45" t="s">
+      <c r="N18" s="45"/>
+      <c r="O18" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="P18" s="45"/>
-      <c r="Q18" s="46"/>
+      <c r="P18" s="46"/>
+      <c r="Q18" s="47"/>
     </row>
     <row r="19" spans="1:17">
-      <c r="A19" s="67" t="s">
+      <c r="A19" s="68" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="67"/>
-      <c r="C19" s="41" t="s">
+      <c r="B19" s="68"/>
+      <c r="C19" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="D19" s="41"/>
-      <c r="E19" s="41"/>
-      <c r="F19" s="41"/>
-      <c r="G19" s="68" t="s">
+      <c r="D19" s="42"/>
+      <c r="E19" s="42"/>
+      <c r="F19" s="42"/>
+      <c r="G19" s="69" t="s">
         <v>27</v>
       </c>
-      <c r="H19" s="68"/>
-      <c r="I19" s="68"/>
-      <c r="J19" s="68"/>
-      <c r="K19" s="68"/>
-      <c r="L19" s="68"/>
-      <c r="M19" s="69">
+      <c r="H19" s="69"/>
+      <c r="I19" s="69"/>
+      <c r="J19" s="69"/>
+      <c r="K19" s="69"/>
+      <c r="L19" s="69"/>
+      <c r="M19" s="70">
         <f>M17-M18</f>
         <v>0</v>
       </c>
-      <c r="N19" s="44"/>
-      <c r="O19" s="45" t="s">
+      <c r="N19" s="45"/>
+      <c r="O19" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="P19" s="45"/>
-      <c r="Q19" s="46"/>
+      <c r="P19" s="46"/>
+      <c r="Q19" s="47"/>
     </row>
     <row r="20" spans="1:17">
-      <c r="A20" s="47" t="s">
+      <c r="A20" s="48" t="s">
         <v>28</v>
       </c>
-      <c r="B20" s="48"/>
-      <c r="C20" s="41" t="s">
+      <c r="B20" s="49"/>
+      <c r="C20" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="D20" s="41"/>
-      <c r="E20" s="41"/>
-      <c r="F20" s="41"/>
-      <c r="G20" s="41"/>
-      <c r="H20" s="41"/>
-      <c r="I20" s="41"/>
-      <c r="J20" s="41"/>
-      <c r="K20" s="41"/>
-      <c r="L20" s="41"/>
-      <c r="M20" s="41"/>
-      <c r="N20" s="41"/>
-      <c r="O20" s="41"/>
-      <c r="P20" s="41"/>
-      <c r="Q20" s="41"/>
+      <c r="D20" s="42"/>
+      <c r="E20" s="42"/>
+      <c r="F20" s="42"/>
+      <c r="G20" s="42"/>
+      <c r="H20" s="42"/>
+      <c r="I20" s="42"/>
+      <c r="J20" s="42"/>
+      <c r="K20" s="42"/>
+      <c r="L20" s="42"/>
+      <c r="M20" s="42"/>
+      <c r="N20" s="42"/>
+      <c r="O20" s="42"/>
+      <c r="P20" s="42"/>
+      <c r="Q20" s="42"/>
     </row>
     <row r="21" spans="1:17" ht="15" customHeight="1">
-      <c r="A21" s="49" t="s">
+      <c r="A21" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="B21" s="50"/>
-      <c r="C21" s="53" t="s">
+      <c r="B21" s="51"/>
+      <c r="C21" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="D21" s="53"/>
-      <c r="E21" s="53"/>
-      <c r="F21" s="53"/>
-      <c r="G21" s="53"/>
-      <c r="H21" s="53"/>
-      <c r="I21" s="53"/>
-      <c r="J21" s="53"/>
-      <c r="K21" s="53"/>
-      <c r="L21" s="53"/>
-      <c r="M21" s="53"/>
-      <c r="N21" s="53"/>
-      <c r="O21" s="53"/>
-      <c r="P21" s="53"/>
-      <c r="Q21" s="53"/>
+      <c r="D21" s="54"/>
+      <c r="E21" s="54"/>
+      <c r="F21" s="54"/>
+      <c r="G21" s="54"/>
+      <c r="H21" s="54"/>
+      <c r="I21" s="54"/>
+      <c r="J21" s="54"/>
+      <c r="K21" s="54"/>
+      <c r="L21" s="54"/>
+      <c r="M21" s="54"/>
+      <c r="N21" s="54"/>
+      <c r="O21" s="54"/>
+      <c r="P21" s="54"/>
+      <c r="Q21" s="54"/>
     </row>
     <row r="22" spans="1:17" ht="14.25" customHeight="1">
-      <c r="A22" s="51"/>
-      <c r="B22" s="52"/>
-      <c r="C22" s="53"/>
-      <c r="D22" s="53"/>
-      <c r="E22" s="53"/>
-      <c r="F22" s="53"/>
-      <c r="G22" s="53"/>
-      <c r="H22" s="53"/>
-      <c r="I22" s="53"/>
-      <c r="J22" s="53"/>
-      <c r="K22" s="53"/>
-      <c r="L22" s="53"/>
-      <c r="M22" s="53"/>
-      <c r="N22" s="53"/>
-      <c r="O22" s="53"/>
-      <c r="P22" s="53"/>
-      <c r="Q22" s="53"/>
+      <c r="A22" s="52"/>
+      <c r="B22" s="53"/>
+      <c r="C22" s="54"/>
+      <c r="D22" s="54"/>
+      <c r="E22" s="54"/>
+      <c r="F22" s="54"/>
+      <c r="G22" s="54"/>
+      <c r="H22" s="54"/>
+      <c r="I22" s="54"/>
+      <c r="J22" s="54"/>
+      <c r="K22" s="54"/>
+      <c r="L22" s="54"/>
+      <c r="M22" s="54"/>
+      <c r="N22" s="54"/>
+      <c r="O22" s="54"/>
+      <c r="P22" s="54"/>
+      <c r="Q22" s="54"/>
     </row>
     <row r="24" spans="1:17" ht="31.5" customHeight="1">
-      <c r="A24" s="35" t="s">
+      <c r="A24" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="35"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="35"/>
-      <c r="E24" s="35"/>
-      <c r="F24" s="35"/>
-      <c r="G24" s="35"/>
-      <c r="H24" s="35"/>
-      <c r="I24" s="35"/>
-      <c r="J24" s="35"/>
-      <c r="K24" s="35"/>
-      <c r="L24" s="35"/>
-      <c r="M24" s="35"/>
-      <c r="N24" s="35"/>
-      <c r="O24" s="35"/>
-      <c r="P24" s="35"/>
-      <c r="Q24" s="35"/>
+      <c r="B24" s="36"/>
+      <c r="C24" s="36"/>
+      <c r="D24" s="36"/>
+      <c r="E24" s="36"/>
+      <c r="F24" s="36"/>
+      <c r="G24" s="36"/>
+      <c r="H24" s="36"/>
+      <c r="I24" s="36"/>
+      <c r="J24" s="36"/>
+      <c r="K24" s="36"/>
+      <c r="L24" s="36"/>
+      <c r="M24" s="36"/>
+      <c r="N24" s="36"/>
+      <c r="O24" s="36"/>
+      <c r="P24" s="36"/>
+      <c r="Q24" s="36"/>
     </row>
     <row r="26" spans="1:17">
-      <c r="A26" s="38" t="s">
+      <c r="A26" s="39" t="s">
         <v>33</v>
       </c>
-      <c r="B26" s="38"/>
-      <c r="C26" s="38"/>
-      <c r="F26" s="38" t="s">
+      <c r="B26" s="39"/>
+      <c r="C26" s="39"/>
+      <c r="F26" s="39" t="s">
         <v>31</v>
       </c>
-      <c r="G26" s="38"/>
-      <c r="H26" s="38"/>
-      <c r="I26" s="38"/>
-      <c r="J26" s="38"/>
-      <c r="K26" s="38"/>
-      <c r="L26" s="38"/>
-      <c r="M26" s="38"/>
-      <c r="N26" s="38"/>
-      <c r="O26" s="38"/>
-      <c r="P26" s="38"/>
-      <c r="Q26" s="38"/>
+      <c r="G26" s="39"/>
+      <c r="H26" s="39"/>
+      <c r="I26" s="39"/>
+      <c r="J26" s="39"/>
+      <c r="K26" s="39"/>
+      <c r="L26" s="39"/>
+      <c r="M26" s="39"/>
+      <c r="N26" s="39"/>
+      <c r="O26" s="39"/>
+      <c r="P26" s="39"/>
+      <c r="Q26" s="39"/>
     </row>
     <row r="27" spans="1:17" ht="57.75" customHeight="1">
-      <c r="A27" s="36"/>
-      <c r="B27" s="36"/>
-      <c r="C27" s="36"/>
-      <c r="F27" s="36"/>
-      <c r="G27" s="36"/>
-      <c r="H27" s="36"/>
-      <c r="I27" s="36"/>
-      <c r="J27" s="36"/>
-      <c r="K27" s="36"/>
-      <c r="L27" s="36"/>
-      <c r="M27" s="36"/>
-      <c r="N27" s="36"/>
-      <c r="O27" s="36"/>
-      <c r="P27" s="36"/>
-      <c r="Q27" s="36"/>
+      <c r="A27" s="37"/>
+      <c r="B27" s="37"/>
+      <c r="C27" s="37"/>
+      <c r="F27" s="37"/>
+      <c r="G27" s="37"/>
+      <c r="H27" s="37"/>
+      <c r="I27" s="37"/>
+      <c r="J27" s="37"/>
+      <c r="K27" s="37"/>
+      <c r="L27" s="37"/>
+      <c r="M27" s="37"/>
+      <c r="N27" s="37"/>
+      <c r="O27" s="37"/>
+      <c r="P27" s="37"/>
+      <c r="Q27" s="37"/>
     </row>
     <row r="28" spans="1:17" s="16" customFormat="1">
-      <c r="A28" s="37" t="s">
+      <c r="A28" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="B28" s="37"/>
-      <c r="C28" s="37"/>
-      <c r="F28" s="37"/>
-      <c r="G28" s="37"/>
-      <c r="H28" s="37"/>
-      <c r="I28" s="37"/>
-      <c r="J28" s="37"/>
-      <c r="K28" s="37"/>
-      <c r="L28" s="37"/>
-      <c r="M28" s="37"/>
-      <c r="N28" s="37"/>
-      <c r="O28" s="37"/>
-      <c r="P28" s="37"/>
-      <c r="Q28" s="37"/>
-    </row>
+      <c r="B28" s="38"/>
+      <c r="C28" s="38"/>
+      <c r="F28" s="38"/>
+      <c r="G28" s="38"/>
+      <c r="H28" s="38"/>
+      <c r="I28" s="38"/>
+      <c r="J28" s="38"/>
+      <c r="K28" s="38"/>
+      <c r="L28" s="38"/>
+      <c r="M28" s="38"/>
+      <c r="N28" s="38"/>
+      <c r="O28" s="38"/>
+      <c r="P28" s="38"/>
+      <c r="Q28" s="38"/>
+    </row>
+    <row r="34" spans="1:17" ht="10" customHeight="1"/>
+    <row r="35" spans="1:17" hidden="1"/>
     <row r="36" spans="1:17" ht="16.5" customHeight="1"/>
     <row r="37" spans="1:17" ht="39.75" customHeight="1">
-      <c r="A37" s="34" t="s">
+      <c r="A37" s="35" t="s">
         <v>32</v>
       </c>
-      <c r="B37" s="34"/>
-      <c r="C37" s="34"/>
-      <c r="D37" s="34"/>
-      <c r="E37" s="34"/>
-      <c r="F37" s="34"/>
-      <c r="G37" s="34"/>
-      <c r="H37" s="34"/>
-      <c r="I37" s="34"/>
-      <c r="J37" s="34"/>
-      <c r="K37" s="34"/>
-      <c r="L37" s="34"/>
-      <c r="M37" s="34"/>
-      <c r="N37" s="34"/>
-      <c r="O37" s="34"/>
-      <c r="P37" s="34"/>
-      <c r="Q37" s="34"/>
+      <c r="B37" s="35"/>
+      <c r="C37" s="35"/>
+      <c r="D37" s="35"/>
+      <c r="E37" s="35"/>
+      <c r="F37" s="35"/>
+      <c r="G37" s="35"/>
+      <c r="H37" s="35"/>
+      <c r="I37" s="35"/>
+      <c r="J37" s="35"/>
+      <c r="K37" s="35"/>
+      <c r="L37" s="35"/>
+      <c r="M37" s="35"/>
+      <c r="N37" s="35"/>
+      <c r="O37" s="35"/>
+      <c r="P37" s="35"/>
+      <c r="Q37" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="49">

</xml_diff>

<commit_message>
3.1.11 Se agrega nombre del proyecto al dictamen
</commit_message>
<xml_diff>
--- a/static/plantillas/XXX-XXX-XXX-X-XXX-XXX-XXX DictamenPruebas PRUEBAS.xlsx
+++ b/static/plantillas/XXX-XXX-XXX-X-XXX-XXX-XXX DictamenPruebas PRUEBAS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BID-eduardo.hernande\Desktop\extractor\excel_extractor\static\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA030A52-C14E-4AA9-A931-02201BB29B8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{572668ED-4A2F-42CE-8C7B-B13D5703E9F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{1A5253DA-6AA8-4BED-9DA7-B3D404B25E3E}"/>
   </bookViews>
@@ -900,124 +900,64 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1048,41 +988,101 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1572,12 +1572,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" ht="28.5" customHeight="1">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="41" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
       <c r="E2" s="17" t="s">
         <v>1</v>
       </c>
@@ -1619,79 +1619,79 @@
       </c>
     </row>
     <row r="3" spans="1:17">
-      <c r="A3" s="46" t="s">
+      <c r="A3" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="46"/>
-      <c r="I3" s="46"/>
-      <c r="J3" s="46"/>
-      <c r="K3" s="46"/>
-      <c r="L3" s="46"/>
-      <c r="M3" s="46"/>
-      <c r="N3" s="46"/>
-      <c r="O3" s="46"/>
-      <c r="P3" s="46"/>
-      <c r="Q3" s="46"/>
+      <c r="B3" s="42"/>
+      <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="42"/>
+      <c r="G3" s="42"/>
+      <c r="H3" s="42"/>
+      <c r="I3" s="42"/>
+      <c r="J3" s="42"/>
+      <c r="K3" s="42"/>
+      <c r="L3" s="42"/>
+      <c r="M3" s="42"/>
+      <c r="N3" s="42"/>
+      <c r="O3" s="42"/>
+      <c r="P3" s="42"/>
+      <c r="Q3" s="42"/>
     </row>
     <row r="5" spans="1:17" ht="14" customHeight="1">
       <c r="A5" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="91" t="s">
+      <c r="B5" s="43" t="s">
         <v>54</v>
       </c>
-      <c r="C5" s="91"/>
-      <c r="D5" s="91"/>
-      <c r="E5" s="92" t="s">
+      <c r="C5" s="43"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="92"/>
-      <c r="G5" s="92"/>
-      <c r="H5" s="92"/>
-      <c r="I5" s="92"/>
-      <c r="J5" s="93"/>
-      <c r="K5" s="94" t="s">
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
+      <c r="H5" s="44"/>
+      <c r="I5" s="44"/>
+      <c r="J5" s="45"/>
+      <c r="K5" s="46" t="s">
         <v>58</v>
       </c>
-      <c r="L5" s="95"/>
-      <c r="M5" s="95"/>
-      <c r="N5" s="95"/>
-      <c r="O5" s="95"/>
-      <c r="P5" s="95"/>
-      <c r="Q5" s="96"/>
+      <c r="L5" s="47"/>
+      <c r="M5" s="47"/>
+      <c r="N5" s="47"/>
+      <c r="O5" s="47"/>
+      <c r="P5" s="47"/>
+      <c r="Q5" s="48"/>
     </row>
     <row r="6" spans="1:17" ht="18" customHeight="1">
       <c r="A6" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="85" t="s">
+      <c r="B6" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="C6" s="85"/>
-      <c r="D6" s="85"/>
-      <c r="E6" s="86" t="s">
+      <c r="C6" s="35"/>
+      <c r="D6" s="35"/>
+      <c r="E6" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="86"/>
-      <c r="G6" s="86"/>
-      <c r="H6" s="86"/>
-      <c r="I6" s="86"/>
-      <c r="J6" s="87"/>
-      <c r="K6" s="88" t="s">
+      <c r="F6" s="36"/>
+      <c r="G6" s="36"/>
+      <c r="H6" s="36"/>
+      <c r="I6" s="36"/>
+      <c r="J6" s="37"/>
+      <c r="K6" s="38" t="s">
         <v>59</v>
       </c>
-      <c r="L6" s="89"/>
-      <c r="M6" s="89"/>
-      <c r="N6" s="89"/>
-      <c r="O6" s="89"/>
-      <c r="P6" s="89"/>
-      <c r="Q6" s="90"/>
+      <c r="L6" s="39"/>
+      <c r="M6" s="39"/>
+      <c r="N6" s="39"/>
+      <c r="O6" s="39"/>
+      <c r="P6" s="39"/>
+      <c r="Q6" s="40"/>
     </row>
     <row r="7" spans="1:17">
       <c r="A7" s="3" t="s">
@@ -1708,18 +1708,18 @@
       <c r="H7" s="7"/>
       <c r="I7" s="7"/>
       <c r="J7" s="8"/>
-      <c r="K7" s="73" t="s">
+      <c r="K7" s="51" t="s">
         <v>9</v>
       </c>
-      <c r="L7" s="74"/>
-      <c r="M7" s="58" t="s">
+      <c r="L7" s="52"/>
+      <c r="M7" s="53" t="s">
         <v>44</v>
       </c>
-      <c r="N7" s="60"/>
-      <c r="O7" s="73" t="s">
+      <c r="N7" s="54"/>
+      <c r="O7" s="51" t="s">
         <v>10</v>
       </c>
-      <c r="P7" s="74"/>
+      <c r="P7" s="52"/>
       <c r="Q7" s="9" t="s">
         <v>44</v>
       </c>
@@ -1728,124 +1728,124 @@
       <c r="A8" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="75" t="s">
+      <c r="B8" s="55" t="s">
         <v>45</v>
       </c>
-      <c r="C8" s="75"/>
-      <c r="D8" s="75"/>
-      <c r="E8" s="75"/>
-      <c r="F8" s="75"/>
-      <c r="G8" s="75"/>
-      <c r="H8" s="75"/>
-      <c r="I8" s="75"/>
-      <c r="J8" s="75"/>
-      <c r="K8" s="75"/>
-      <c r="L8" s="75"/>
-      <c r="M8" s="75"/>
-      <c r="N8" s="75"/>
-      <c r="O8" s="75"/>
-      <c r="P8" s="75"/>
-      <c r="Q8" s="75"/>
+      <c r="C8" s="55"/>
+      <c r="D8" s="55"/>
+      <c r="E8" s="55"/>
+      <c r="F8" s="55"/>
+      <c r="G8" s="55"/>
+      <c r="H8" s="55"/>
+      <c r="I8" s="55"/>
+      <c r="J8" s="55"/>
+      <c r="K8" s="55"/>
+      <c r="L8" s="55"/>
+      <c r="M8" s="55"/>
+      <c r="N8" s="55"/>
+      <c r="O8" s="55"/>
+      <c r="P8" s="55"/>
+      <c r="Q8" s="55"/>
     </row>
     <row r="9" spans="1:17">
-      <c r="A9" s="71" t="s">
+      <c r="A9" s="49" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="76"/>
-      <c r="C9" s="77" t="s">
+      <c r="B9" s="56"/>
+      <c r="C9" s="57" t="s">
         <v>45</v>
       </c>
-      <c r="D9" s="77"/>
-      <c r="E9" s="77"/>
-      <c r="F9" s="77"/>
-      <c r="G9" s="77"/>
-      <c r="H9" s="77"/>
-      <c r="I9" s="77"/>
-      <c r="J9" s="77"/>
-      <c r="K9" s="77"/>
-      <c r="L9" s="77"/>
-      <c r="M9" s="77"/>
-      <c r="N9" s="77"/>
-      <c r="O9" s="77"/>
-      <c r="P9" s="77"/>
-      <c r="Q9" s="78"/>
+      <c r="D9" s="57"/>
+      <c r="E9" s="57"/>
+      <c r="F9" s="57"/>
+      <c r="G9" s="57"/>
+      <c r="H9" s="57"/>
+      <c r="I9" s="57"/>
+      <c r="J9" s="57"/>
+      <c r="K9" s="57"/>
+      <c r="L9" s="57"/>
+      <c r="M9" s="57"/>
+      <c r="N9" s="57"/>
+      <c r="O9" s="57"/>
+      <c r="P9" s="57"/>
+      <c r="Q9" s="58"/>
     </row>
     <row r="10" spans="1:17">
-      <c r="A10" s="79" t="s">
+      <c r="A10" s="59" t="s">
         <v>13</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="80" t="s">
+      <c r="C10" s="60" t="s">
         <v>44</v>
       </c>
-      <c r="D10" s="80"/>
-      <c r="E10" s="80"/>
-      <c r="F10" s="80"/>
-      <c r="G10" s="80"/>
-      <c r="H10" s="80"/>
-      <c r="I10" s="80"/>
-      <c r="J10" s="80"/>
-      <c r="K10" s="80"/>
-      <c r="L10" s="80"/>
-      <c r="M10" s="80"/>
-      <c r="N10" s="80"/>
-      <c r="O10" s="80"/>
-      <c r="P10" s="80"/>
-      <c r="Q10" s="80"/>
+      <c r="D10" s="60"/>
+      <c r="E10" s="60"/>
+      <c r="F10" s="60"/>
+      <c r="G10" s="60"/>
+      <c r="H10" s="60"/>
+      <c r="I10" s="60"/>
+      <c r="J10" s="60"/>
+      <c r="K10" s="60"/>
+      <c r="L10" s="60"/>
+      <c r="M10" s="60"/>
+      <c r="N10" s="60"/>
+      <c r="O10" s="60"/>
+      <c r="P10" s="60"/>
+      <c r="Q10" s="60"/>
     </row>
     <row r="11" spans="1:17">
-      <c r="A11" s="79"/>
+      <c r="A11" s="59"/>
       <c r="B11" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="80" t="s">
+      <c r="C11" s="60" t="s">
         <v>44</v>
       </c>
-      <c r="D11" s="80"/>
-      <c r="E11" s="80"/>
-      <c r="F11" s="80"/>
-      <c r="G11" s="80"/>
-      <c r="H11" s="80"/>
-      <c r="I11" s="80"/>
-      <c r="J11" s="80"/>
-      <c r="K11" s="80"/>
-      <c r="L11" s="80"/>
-      <c r="M11" s="80"/>
-      <c r="N11" s="80"/>
-      <c r="O11" s="80"/>
-      <c r="P11" s="80"/>
-      <c r="Q11" s="80"/>
+      <c r="D11" s="60"/>
+      <c r="E11" s="60"/>
+      <c r="F11" s="60"/>
+      <c r="G11" s="60"/>
+      <c r="H11" s="60"/>
+      <c r="I11" s="60"/>
+      <c r="J11" s="60"/>
+      <c r="K11" s="60"/>
+      <c r="L11" s="60"/>
+      <c r="M11" s="60"/>
+      <c r="N11" s="60"/>
+      <c r="O11" s="60"/>
+      <c r="P11" s="60"/>
+      <c r="Q11" s="60"/>
     </row>
     <row r="12" spans="1:17">
       <c r="A12" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="81" t="s">
+      <c r="B12" s="61" t="s">
         <v>44</v>
       </c>
-      <c r="C12" s="82"/>
-      <c r="D12" s="82"/>
-      <c r="E12" s="82"/>
-      <c r="F12" s="82"/>
-      <c r="G12" s="82"/>
-      <c r="H12" s="82"/>
-      <c r="I12" s="82"/>
-      <c r="J12" s="82"/>
-      <c r="K12" s="82"/>
-      <c r="L12" s="82"/>
-      <c r="M12" s="82"/>
-      <c r="N12" s="82"/>
-      <c r="O12" s="82"/>
-      <c r="P12" s="82"/>
-      <c r="Q12" s="83"/>
+      <c r="C12" s="62"/>
+      <c r="D12" s="62"/>
+      <c r="E12" s="62"/>
+      <c r="F12" s="62"/>
+      <c r="G12" s="62"/>
+      <c r="H12" s="62"/>
+      <c r="I12" s="62"/>
+      <c r="J12" s="62"/>
+      <c r="K12" s="62"/>
+      <c r="L12" s="62"/>
+      <c r="M12" s="62"/>
+      <c r="N12" s="62"/>
+      <c r="O12" s="62"/>
+      <c r="P12" s="62"/>
+      <c r="Q12" s="63"/>
     </row>
     <row r="13" spans="1:17">
-      <c r="A13" s="71" t="s">
+      <c r="A13" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="84"/>
+      <c r="B13" s="64"/>
       <c r="C13" s="12" t="s">
         <v>44</v>
       </c>
@@ -1865,10 +1865,10 @@
       <c r="Q13" s="14"/>
     </row>
     <row r="14" spans="1:17">
-      <c r="A14" s="71" t="s">
+      <c r="A14" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="72"/>
+      <c r="B14" s="50"/>
       <c r="C14" s="15" t="s">
         <v>44</v>
       </c>
@@ -1891,321 +1891,315 @@
       <c r="A15" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="42" t="s">
+      <c r="B15" s="67" t="s">
         <v>44</v>
       </c>
-      <c r="C15" s="42"/>
-      <c r="D15" s="42"/>
-      <c r="E15" s="42"/>
-      <c r="F15" s="42"/>
-      <c r="G15" s="42"/>
-      <c r="H15" s="42"/>
-      <c r="I15" s="42"/>
-      <c r="J15" s="42"/>
-      <c r="K15" s="42"/>
-      <c r="L15" s="42"/>
-      <c r="M15" s="42"/>
-      <c r="N15" s="42"/>
-      <c r="O15" s="42"/>
-      <c r="P15" s="42"/>
-      <c r="Q15" s="42"/>
+      <c r="C15" s="67"/>
+      <c r="D15" s="67"/>
+      <c r="E15" s="67"/>
+      <c r="F15" s="67"/>
+      <c r="G15" s="67"/>
+      <c r="H15" s="67"/>
+      <c r="I15" s="67"/>
+      <c r="J15" s="67"/>
+      <c r="K15" s="67"/>
+      <c r="L15" s="67"/>
+      <c r="M15" s="67"/>
+      <c r="N15" s="67"/>
+      <c r="O15" s="67"/>
+      <c r="P15" s="67"/>
+      <c r="Q15" s="67"/>
     </row>
     <row r="16" spans="1:17">
-      <c r="A16" s="44" t="s">
+      <c r="A16" s="73" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="55"/>
-      <c r="C16" s="56"/>
-      <c r="D16" s="56"/>
-      <c r="E16" s="56"/>
-      <c r="F16" s="56"/>
-      <c r="G16" s="55"/>
-      <c r="H16" s="55"/>
-      <c r="I16" s="55"/>
-      <c r="J16" s="55"/>
-      <c r="K16" s="55"/>
-      <c r="L16" s="55"/>
-      <c r="M16" s="56"/>
-      <c r="N16" s="56"/>
-      <c r="O16" s="56"/>
-      <c r="P16" s="56"/>
-      <c r="Q16" s="57"/>
+      <c r="B16" s="74"/>
+      <c r="C16" s="75"/>
+      <c r="D16" s="75"/>
+      <c r="E16" s="75"/>
+      <c r="F16" s="75"/>
+      <c r="G16" s="74"/>
+      <c r="H16" s="74"/>
+      <c r="I16" s="74"/>
+      <c r="J16" s="74"/>
+      <c r="K16" s="74"/>
+      <c r="L16" s="74"/>
+      <c r="M16" s="75"/>
+      <c r="N16" s="75"/>
+      <c r="O16" s="75"/>
+      <c r="P16" s="75"/>
+      <c r="Q16" s="76"/>
     </row>
     <row r="17" spans="1:17">
-      <c r="A17" s="48" t="s">
+      <c r="A17" s="65" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="48"/>
-      <c r="C17" s="58"/>
-      <c r="D17" s="59"/>
-      <c r="E17" s="59"/>
-      <c r="F17" s="60"/>
-      <c r="G17" s="61" t="s">
+      <c r="B17" s="65"/>
+      <c r="C17" s="53"/>
+      <c r="D17" s="77"/>
+      <c r="E17" s="77"/>
+      <c r="F17" s="54"/>
+      <c r="G17" s="78" t="s">
         <v>22</v>
       </c>
-      <c r="H17" s="62"/>
-      <c r="I17" s="62"/>
-      <c r="J17" s="62"/>
-      <c r="K17" s="62"/>
-      <c r="L17" s="63"/>
-      <c r="M17" s="64">
+      <c r="H17" s="79"/>
+      <c r="I17" s="79"/>
+      <c r="J17" s="79"/>
+      <c r="K17" s="79"/>
+      <c r="L17" s="80"/>
+      <c r="M17" s="81">
         <v>16</v>
       </c>
-      <c r="N17" s="65"/>
-      <c r="O17" s="66" t="s">
+      <c r="N17" s="82"/>
+      <c r="O17" s="83" t="s">
         <v>23</v>
       </c>
-      <c r="P17" s="66"/>
-      <c r="Q17" s="67"/>
+      <c r="P17" s="83"/>
+      <c r="Q17" s="84"/>
     </row>
     <row r="18" spans="1:17">
-      <c r="A18" s="40" t="s">
+      <c r="A18" s="90" t="s">
         <v>24</v>
       </c>
-      <c r="B18" s="41"/>
-      <c r="C18" s="42">
+      <c r="B18" s="91"/>
+      <c r="C18" s="67">
         <v>1</v>
       </c>
-      <c r="D18" s="42"/>
-      <c r="E18" s="42"/>
-      <c r="F18" s="43"/>
-      <c r="G18" s="44" t="s">
+      <c r="D18" s="67"/>
+      <c r="E18" s="67"/>
+      <c r="F18" s="92"/>
+      <c r="G18" s="73" t="s">
         <v>25</v>
       </c>
-      <c r="H18" s="44"/>
-      <c r="I18" s="44"/>
-      <c r="J18" s="44"/>
-      <c r="K18" s="44"/>
-      <c r="L18" s="44"/>
-      <c r="M18" s="45">
+      <c r="H18" s="73"/>
+      <c r="I18" s="73"/>
+      <c r="J18" s="73"/>
+      <c r="K18" s="73"/>
+      <c r="L18" s="73"/>
+      <c r="M18" s="88">
         <v>16</v>
       </c>
-      <c r="N18" s="45"/>
-      <c r="O18" s="46" t="s">
+      <c r="N18" s="88"/>
+      <c r="O18" s="42" t="s">
         <v>23</v>
       </c>
-      <c r="P18" s="46"/>
-      <c r="Q18" s="47"/>
+      <c r="P18" s="42"/>
+      <c r="Q18" s="89"/>
     </row>
     <row r="19" spans="1:17">
-      <c r="A19" s="68" t="s">
+      <c r="A19" s="85" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="68"/>
-      <c r="C19" s="42" t="s">
+      <c r="B19" s="85"/>
+      <c r="C19" s="67" t="s">
         <v>46</v>
       </c>
-      <c r="D19" s="42"/>
-      <c r="E19" s="42"/>
-      <c r="F19" s="42"/>
-      <c r="G19" s="69" t="s">
+      <c r="D19" s="67"/>
+      <c r="E19" s="67"/>
+      <c r="F19" s="67"/>
+      <c r="G19" s="86" t="s">
         <v>27</v>
       </c>
-      <c r="H19" s="69"/>
-      <c r="I19" s="69"/>
-      <c r="J19" s="69"/>
-      <c r="K19" s="69"/>
-      <c r="L19" s="69"/>
-      <c r="M19" s="70">
+      <c r="H19" s="86"/>
+      <c r="I19" s="86"/>
+      <c r="J19" s="86"/>
+      <c r="K19" s="86"/>
+      <c r="L19" s="86"/>
+      <c r="M19" s="87">
         <f>M17-M18</f>
         <v>0</v>
       </c>
-      <c r="N19" s="45"/>
-      <c r="O19" s="46" t="s">
+      <c r="N19" s="88"/>
+      <c r="O19" s="42" t="s">
         <v>23</v>
       </c>
-      <c r="P19" s="46"/>
-      <c r="Q19" s="47"/>
+      <c r="P19" s="42"/>
+      <c r="Q19" s="89"/>
     </row>
     <row r="20" spans="1:17">
-      <c r="A20" s="48" t="s">
+      <c r="A20" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="B20" s="49"/>
-      <c r="C20" s="42" t="s">
+      <c r="B20" s="66"/>
+      <c r="C20" s="67" t="s">
         <v>46</v>
       </c>
-      <c r="D20" s="42"/>
-      <c r="E20" s="42"/>
-      <c r="F20" s="42"/>
-      <c r="G20" s="42"/>
-      <c r="H20" s="42"/>
-      <c r="I20" s="42"/>
-      <c r="J20" s="42"/>
-      <c r="K20" s="42"/>
-      <c r="L20" s="42"/>
-      <c r="M20" s="42"/>
-      <c r="N20" s="42"/>
-      <c r="O20" s="42"/>
-      <c r="P20" s="42"/>
-      <c r="Q20" s="42"/>
+      <c r="D20" s="67"/>
+      <c r="E20" s="67"/>
+      <c r="F20" s="67"/>
+      <c r="G20" s="67"/>
+      <c r="H20" s="67"/>
+      <c r="I20" s="67"/>
+      <c r="J20" s="67"/>
+      <c r="K20" s="67"/>
+      <c r="L20" s="67"/>
+      <c r="M20" s="67"/>
+      <c r="N20" s="67"/>
+      <c r="O20" s="67"/>
+      <c r="P20" s="67"/>
+      <c r="Q20" s="67"/>
     </row>
     <row r="21" spans="1:17" ht="15" customHeight="1">
-      <c r="A21" s="50" t="s">
+      <c r="A21" s="68" t="s">
         <v>29</v>
       </c>
-      <c r="B21" s="51"/>
-      <c r="C21" s="54" t="s">
+      <c r="B21" s="69"/>
+      <c r="C21" s="72" t="s">
         <v>47</v>
       </c>
-      <c r="D21" s="54"/>
-      <c r="E21" s="54"/>
-      <c r="F21" s="54"/>
-      <c r="G21" s="54"/>
-      <c r="H21" s="54"/>
-      <c r="I21" s="54"/>
-      <c r="J21" s="54"/>
-      <c r="K21" s="54"/>
-      <c r="L21" s="54"/>
-      <c r="M21" s="54"/>
-      <c r="N21" s="54"/>
-      <c r="O21" s="54"/>
-      <c r="P21" s="54"/>
-      <c r="Q21" s="54"/>
+      <c r="D21" s="72"/>
+      <c r="E21" s="72"/>
+      <c r="F21" s="72"/>
+      <c r="G21" s="72"/>
+      <c r="H21" s="72"/>
+      <c r="I21" s="72"/>
+      <c r="J21" s="72"/>
+      <c r="K21" s="72"/>
+      <c r="L21" s="72"/>
+      <c r="M21" s="72"/>
+      <c r="N21" s="72"/>
+      <c r="O21" s="72"/>
+      <c r="P21" s="72"/>
+      <c r="Q21" s="72"/>
     </row>
     <row r="22" spans="1:17" ht="14.25" customHeight="1">
-      <c r="A22" s="52"/>
-      <c r="B22" s="53"/>
-      <c r="C22" s="54"/>
-      <c r="D22" s="54"/>
-      <c r="E22" s="54"/>
-      <c r="F22" s="54"/>
-      <c r="G22" s="54"/>
-      <c r="H22" s="54"/>
-      <c r="I22" s="54"/>
-      <c r="J22" s="54"/>
-      <c r="K22" s="54"/>
-      <c r="L22" s="54"/>
-      <c r="M22" s="54"/>
-      <c r="N22" s="54"/>
-      <c r="O22" s="54"/>
-      <c r="P22" s="54"/>
-      <c r="Q22" s="54"/>
+      <c r="A22" s="70"/>
+      <c r="B22" s="71"/>
+      <c r="C22" s="72"/>
+      <c r="D22" s="72"/>
+      <c r="E22" s="72"/>
+      <c r="F22" s="72"/>
+      <c r="G22" s="72"/>
+      <c r="H22" s="72"/>
+      <c r="I22" s="72"/>
+      <c r="J22" s="72"/>
+      <c r="K22" s="72"/>
+      <c r="L22" s="72"/>
+      <c r="M22" s="72"/>
+      <c r="N22" s="72"/>
+      <c r="O22" s="72"/>
+      <c r="P22" s="72"/>
+      <c r="Q22" s="72"/>
     </row>
     <row r="24" spans="1:17" ht="31.5" customHeight="1">
-      <c r="A24" s="36" t="s">
+      <c r="A24" s="41" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="36"/>
-      <c r="C24" s="36"/>
-      <c r="D24" s="36"/>
-      <c r="E24" s="36"/>
-      <c r="F24" s="36"/>
-      <c r="G24" s="36"/>
-      <c r="H24" s="36"/>
-      <c r="I24" s="36"/>
-      <c r="J24" s="36"/>
-      <c r="K24" s="36"/>
-      <c r="L24" s="36"/>
-      <c r="M24" s="36"/>
-      <c r="N24" s="36"/>
-      <c r="O24" s="36"/>
-      <c r="P24" s="36"/>
-      <c r="Q24" s="36"/>
+      <c r="B24" s="41"/>
+      <c r="C24" s="41"/>
+      <c r="D24" s="41"/>
+      <c r="E24" s="41"/>
+      <c r="F24" s="41"/>
+      <c r="G24" s="41"/>
+      <c r="H24" s="41"/>
+      <c r="I24" s="41"/>
+      <c r="J24" s="41"/>
+      <c r="K24" s="41"/>
+      <c r="L24" s="41"/>
+      <c r="M24" s="41"/>
+      <c r="N24" s="41"/>
+      <c r="O24" s="41"/>
+      <c r="P24" s="41"/>
+      <c r="Q24" s="41"/>
     </row>
     <row r="26" spans="1:17">
-      <c r="A26" s="39" t="s">
+      <c r="A26" s="96" t="s">
         <v>33</v>
       </c>
-      <c r="B26" s="39"/>
-      <c r="C26" s="39"/>
-      <c r="F26" s="39" t="s">
+      <c r="B26" s="96"/>
+      <c r="C26" s="96"/>
+      <c r="F26" s="96" t="s">
         <v>31</v>
       </c>
-      <c r="G26" s="39"/>
-      <c r="H26" s="39"/>
-      <c r="I26" s="39"/>
-      <c r="J26" s="39"/>
-      <c r="K26" s="39"/>
-      <c r="L26" s="39"/>
-      <c r="M26" s="39"/>
-      <c r="N26" s="39"/>
-      <c r="O26" s="39"/>
-      <c r="P26" s="39"/>
-      <c r="Q26" s="39"/>
+      <c r="G26" s="96"/>
+      <c r="H26" s="96"/>
+      <c r="I26" s="96"/>
+      <c r="J26" s="96"/>
+      <c r="K26" s="96"/>
+      <c r="L26" s="96"/>
+      <c r="M26" s="96"/>
+      <c r="N26" s="96"/>
+      <c r="O26" s="96"/>
+      <c r="P26" s="96"/>
+      <c r="Q26" s="96"/>
     </row>
     <row r="27" spans="1:17" ht="57.75" customHeight="1">
-      <c r="A27" s="37"/>
-      <c r="B27" s="37"/>
-      <c r="C27" s="37"/>
-      <c r="F27" s="37"/>
-      <c r="G27" s="37"/>
-      <c r="H27" s="37"/>
-      <c r="I27" s="37"/>
-      <c r="J27" s="37"/>
-      <c r="K27" s="37"/>
-      <c r="L27" s="37"/>
-      <c r="M27" s="37"/>
-      <c r="N27" s="37"/>
-      <c r="O27" s="37"/>
-      <c r="P27" s="37"/>
-      <c r="Q27" s="37"/>
+      <c r="A27" s="94"/>
+      <c r="B27" s="94"/>
+      <c r="C27" s="94"/>
+      <c r="F27" s="94"/>
+      <c r="G27" s="94"/>
+      <c r="H27" s="94"/>
+      <c r="I27" s="94"/>
+      <c r="J27" s="94"/>
+      <c r="K27" s="94"/>
+      <c r="L27" s="94"/>
+      <c r="M27" s="94"/>
+      <c r="N27" s="94"/>
+      <c r="O27" s="94"/>
+      <c r="P27" s="94"/>
+      <c r="Q27" s="94"/>
     </row>
     <row r="28" spans="1:17" s="16" customFormat="1">
-      <c r="A28" s="38" t="s">
+      <c r="A28" s="95" t="s">
         <v>57</v>
       </c>
-      <c r="B28" s="38"/>
-      <c r="C28" s="38"/>
-      <c r="F28" s="38"/>
-      <c r="G28" s="38"/>
-      <c r="H28" s="38"/>
-      <c r="I28" s="38"/>
-      <c r="J28" s="38"/>
-      <c r="K28" s="38"/>
-      <c r="L28" s="38"/>
-      <c r="M28" s="38"/>
-      <c r="N28" s="38"/>
-      <c r="O28" s="38"/>
-      <c r="P28" s="38"/>
-      <c r="Q28" s="38"/>
-    </row>
-    <row r="34" spans="1:17" ht="10" customHeight="1"/>
-    <row r="35" spans="1:17" hidden="1"/>
+      <c r="B28" s="95"/>
+      <c r="C28" s="95"/>
+      <c r="F28" s="95"/>
+      <c r="G28" s="95"/>
+      <c r="H28" s="95"/>
+      <c r="I28" s="95"/>
+      <c r="J28" s="95"/>
+      <c r="K28" s="95"/>
+      <c r="L28" s="95"/>
+      <c r="M28" s="95"/>
+      <c r="N28" s="95"/>
+      <c r="O28" s="95"/>
+      <c r="P28" s="95"/>
+      <c r="Q28" s="95"/>
+    </row>
+    <row r="33" spans="1:17" ht="59" customHeight="1"/>
+    <row r="34" spans="1:17" ht="32" customHeight="1">
+      <c r="A34" s="93" t="s">
+        <v>32</v>
+      </c>
+      <c r="B34" s="93"/>
+      <c r="C34" s="93"/>
+      <c r="D34" s="93"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="93"/>
+      <c r="G34" s="93"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="93"/>
+      <c r="J34" s="93"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="93"/>
+      <c r="M34" s="93"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="93"/>
+      <c r="P34" s="93"/>
+      <c r="Q34" s="93"/>
+    </row>
+    <row r="35" spans="1:17" ht="14.5" customHeight="1"/>
     <row r="36" spans="1:17" ht="16.5" customHeight="1"/>
-    <row r="37" spans="1:17" ht="39.75" customHeight="1">
-      <c r="A37" s="35" t="s">
-        <v>32</v>
-      </c>
-      <c r="B37" s="35"/>
-      <c r="C37" s="35"/>
-      <c r="D37" s="35"/>
-      <c r="E37" s="35"/>
-      <c r="F37" s="35"/>
-      <c r="G37" s="35"/>
-      <c r="H37" s="35"/>
-      <c r="I37" s="35"/>
-      <c r="J37" s="35"/>
-      <c r="K37" s="35"/>
-      <c r="L37" s="35"/>
-      <c r="M37" s="35"/>
-      <c r="N37" s="35"/>
-      <c r="O37" s="35"/>
-      <c r="P37" s="35"/>
-      <c r="Q37" s="35"/>
-    </row>
+    <row r="37" spans="1:17" ht="39.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="49">
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="E6:J6"/>
-    <mergeCell ref="K6:Q6"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="E5:J5"/>
-    <mergeCell ref="K5:Q5"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="K7:L7"/>
-    <mergeCell ref="M7:N7"/>
-    <mergeCell ref="O7:P7"/>
-    <mergeCell ref="B8:Q8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C9:Q9"/>
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="C10:Q10"/>
-    <mergeCell ref="C11:Q11"/>
-    <mergeCell ref="B12:Q12"/>
-    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A34:Q34"/>
+    <mergeCell ref="A24:Q24"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="F27:Q27"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="F28:Q28"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="F26:Q26"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="C18:F18"/>
+    <mergeCell ref="G18:L18"/>
+    <mergeCell ref="M18:N18"/>
+    <mergeCell ref="O18:Q18"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="C20:Q20"/>
     <mergeCell ref="A21:B22"/>
@@ -2222,19 +2216,26 @@
     <mergeCell ref="G19:L19"/>
     <mergeCell ref="M19:N19"/>
     <mergeCell ref="O19:Q19"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="C18:F18"/>
-    <mergeCell ref="G18:L18"/>
-    <mergeCell ref="M18:N18"/>
-    <mergeCell ref="O18:Q18"/>
-    <mergeCell ref="A37:Q37"/>
-    <mergeCell ref="A24:Q24"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="F27:Q27"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="F28:Q28"/>
-    <mergeCell ref="A26:C26"/>
-    <mergeCell ref="F26:Q26"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="O7:P7"/>
+    <mergeCell ref="B8:Q8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C9:Q9"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="C10:Q10"/>
+    <mergeCell ref="C11:Q11"/>
+    <mergeCell ref="B12:Q12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="E6:J6"/>
+    <mergeCell ref="K6:Q6"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A3:Q3"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="E5:J5"/>
+    <mergeCell ref="K5:Q5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.80208333333333337" top="1.5625" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
4.0.6.8 Fix Eliminar dictamen
</commit_message>
<xml_diff>
--- a/static/plantillas/XXX-XXX-XXX-X-XXX-XXX-XXX DictamenPruebas PRUEBAS.xlsx
+++ b/static/plantillas/XXX-XXX-XXX-X-XXX-XXX-XXX DictamenPruebas PRUEBAS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BID-eduardo.hernande\Desktop\extractor\excel_extractor\static\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{572668ED-4A2F-42CE-8C7B-B13D5703E9F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B486502-37E8-41ED-82AB-2A0C852EF94E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{1A5253DA-6AA8-4BED-9DA7-B3D404B25E3E}"/>
   </bookViews>
@@ -818,11 +818,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="97">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
@@ -900,6 +899,91 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -918,12 +1002,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -942,147 +1020,65 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1464,66 +1460,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="24"/>
-      <c r="B2" s="25"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
+      <c r="A2" s="23"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="27" t="s">
+      <c r="C3" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="D3" s="27" t="s">
+      <c r="D3" s="26" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="28">
-      <c r="A4" s="29">
+      <c r="A4" s="28">
         <v>45772</v>
       </c>
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="C4" s="30" t="s">
+      <c r="C4" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="D4" s="31" t="s">
+      <c r="D4" s="30" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="28">
-      <c r="A5" s="29">
+      <c r="A5" s="28">
         <v>44774</v>
       </c>
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="30" t="s">
+      <c r="C5" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="D5" s="31" t="s">
+      <c r="D5" s="30" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15.5">
-      <c r="A6" s="28"/>
-      <c r="B6" s="28"/>
-      <c r="C6" s="28"/>
-      <c r="D6" s="28"/>
+      <c r="A6" s="27"/>
+      <c r="B6" s="27"/>
+      <c r="C6" s="27"/>
+      <c r="D6" s="27"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -1572,160 +1568,160 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" ht="28.5" customHeight="1">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="17" t="s">
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="20" t="s">
+      <c r="G2" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="H2" s="19" t="s">
+      <c r="H2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="32" t="s">
+      <c r="I2" s="31" t="s">
         <v>49</v>
       </c>
-      <c r="J2" s="19" t="s">
+      <c r="J2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="K2" s="18" t="s">
+      <c r="K2" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="L2" s="20" t="s">
+      <c r="L2" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="M2" s="18" t="s">
+      <c r="M2" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="N2" s="20" t="s">
+      <c r="N2" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="O2" s="32" t="s">
+      <c r="O2" s="31" t="s">
         <v>52</v>
       </c>
-      <c r="P2" s="20" t="s">
+      <c r="P2" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="Q2" s="33" t="s">
+      <c r="Q2" s="32" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:17">
-      <c r="A3" s="42" t="s">
+      <c r="A3" s="44" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="42"/>
-      <c r="C3" s="42"/>
-      <c r="D3" s="42"/>
-      <c r="E3" s="42"/>
-      <c r="F3" s="42"/>
-      <c r="G3" s="42"/>
-      <c r="H3" s="42"/>
-      <c r="I3" s="42"/>
-      <c r="J3" s="42"/>
-      <c r="K3" s="42"/>
-      <c r="L3" s="42"/>
-      <c r="M3" s="42"/>
-      <c r="N3" s="42"/>
-      <c r="O3" s="42"/>
-      <c r="P3" s="42"/>
-      <c r="Q3" s="42"/>
+      <c r="B3" s="44"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
+      <c r="G3" s="44"/>
+      <c r="H3" s="44"/>
+      <c r="I3" s="44"/>
+      <c r="J3" s="44"/>
+      <c r="K3" s="44"/>
+      <c r="L3" s="44"/>
+      <c r="M3" s="44"/>
+      <c r="N3" s="44"/>
+      <c r="O3" s="44"/>
+      <c r="P3" s="44"/>
+      <c r="Q3" s="44"/>
     </row>
     <row r="5" spans="1:17" ht="14" customHeight="1">
-      <c r="A5" s="34" t="s">
+      <c r="A5" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="43" t="s">
+      <c r="B5" s="69" t="s">
         <v>54</v>
       </c>
-      <c r="C5" s="43"/>
-      <c r="D5" s="43"/>
-      <c r="E5" s="44" t="s">
+      <c r="C5" s="69"/>
+      <c r="D5" s="69"/>
+      <c r="E5" s="70" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="44"/>
-      <c r="G5" s="44"/>
-      <c r="H5" s="44"/>
-      <c r="I5" s="44"/>
-      <c r="J5" s="45"/>
-      <c r="K5" s="46" t="s">
+      <c r="F5" s="70"/>
+      <c r="G5" s="70"/>
+      <c r="H5" s="70"/>
+      <c r="I5" s="70"/>
+      <c r="J5" s="71"/>
+      <c r="K5" s="72" t="s">
         <v>58</v>
       </c>
-      <c r="L5" s="47"/>
-      <c r="M5" s="47"/>
-      <c r="N5" s="47"/>
-      <c r="O5" s="47"/>
-      <c r="P5" s="47"/>
-      <c r="Q5" s="48"/>
+      <c r="L5" s="73"/>
+      <c r="M5" s="73"/>
+      <c r="N5" s="73"/>
+      <c r="O5" s="73"/>
+      <c r="P5" s="73"/>
+      <c r="Q5" s="74"/>
     </row>
     <row r="6" spans="1:17" ht="18" customHeight="1">
-      <c r="A6" s="34" t="s">
+      <c r="A6" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="35" t="s">
+      <c r="B6" s="63" t="s">
         <v>55</v>
       </c>
-      <c r="C6" s="35"/>
-      <c r="D6" s="35"/>
-      <c r="E6" s="36" t="s">
+      <c r="C6" s="63"/>
+      <c r="D6" s="63"/>
+      <c r="E6" s="64" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="36"/>
-      <c r="G6" s="36"/>
-      <c r="H6" s="36"/>
-      <c r="I6" s="36"/>
-      <c r="J6" s="37"/>
-      <c r="K6" s="38" t="s">
+      <c r="F6" s="64"/>
+      <c r="G6" s="64"/>
+      <c r="H6" s="64"/>
+      <c r="I6" s="64"/>
+      <c r="J6" s="65"/>
+      <c r="K6" s="66" t="s">
         <v>59</v>
       </c>
-      <c r="L6" s="39"/>
-      <c r="M6" s="39"/>
-      <c r="N6" s="39"/>
-      <c r="O6" s="39"/>
-      <c r="P6" s="39"/>
-      <c r="Q6" s="40"/>
+      <c r="L6" s="67"/>
+      <c r="M6" s="67"/>
+      <c r="N6" s="67"/>
+      <c r="O6" s="67"/>
+      <c r="P6" s="67"/>
+      <c r="Q6" s="68"/>
     </row>
     <row r="7" spans="1:17">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="77" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="4"/>
-      <c r="C7" s="5" t="s">
+      <c r="B7" s="3"/>
+      <c r="C7" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="D7" s="6"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="51" t="s">
+      <c r="D7" s="5"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="93" t="s">
         <v>9</v>
       </c>
-      <c r="L7" s="52"/>
-      <c r="M7" s="53" t="s">
+      <c r="L7" s="94"/>
+      <c r="M7" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="N7" s="54"/>
-      <c r="O7" s="51" t="s">
+      <c r="N7" s="49"/>
+      <c r="O7" s="93" t="s">
         <v>10</v>
       </c>
-      <c r="P7" s="52"/>
-      <c r="Q7" s="9" t="s">
+      <c r="P7" s="94"/>
+      <c r="Q7" s="8" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:17">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="33" t="s">
         <v>11</v>
       </c>
       <c r="B8" s="55" t="s">
@@ -1748,458 +1744,467 @@
       <c r="Q8" s="55"/>
     </row>
     <row r="9" spans="1:17">
-      <c r="A9" s="49" t="s">
+      <c r="A9" s="78" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="56"/>
-      <c r="C9" s="57" t="s">
+      <c r="B9" s="79"/>
+      <c r="C9" s="56" t="s">
         <v>45</v>
       </c>
-      <c r="D9" s="57"/>
-      <c r="E9" s="57"/>
-      <c r="F9" s="57"/>
-      <c r="G9" s="57"/>
-      <c r="H9" s="57"/>
-      <c r="I9" s="57"/>
-      <c r="J9" s="57"/>
-      <c r="K9" s="57"/>
-      <c r="L9" s="57"/>
-      <c r="M9" s="57"/>
-      <c r="N9" s="57"/>
-      <c r="O9" s="57"/>
-      <c r="P9" s="57"/>
-      <c r="Q9" s="58"/>
+      <c r="D9" s="56"/>
+      <c r="E9" s="56"/>
+      <c r="F9" s="56"/>
+      <c r="G9" s="56"/>
+      <c r="H9" s="56"/>
+      <c r="I9" s="56"/>
+      <c r="J9" s="56"/>
+      <c r="K9" s="56"/>
+      <c r="L9" s="56"/>
+      <c r="M9" s="56"/>
+      <c r="N9" s="56"/>
+      <c r="O9" s="56"/>
+      <c r="P9" s="56"/>
+      <c r="Q9" s="57"/>
     </row>
     <row r="10" spans="1:17">
-      <c r="A10" s="59" t="s">
+      <c r="A10" s="78" t="s">
         <v>13</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="60" t="s">
+      <c r="C10" s="59" t="s">
         <v>44</v>
       </c>
-      <c r="D10" s="60"/>
-      <c r="E10" s="60"/>
-      <c r="F10" s="60"/>
-      <c r="G10" s="60"/>
-      <c r="H10" s="60"/>
-      <c r="I10" s="60"/>
-      <c r="J10" s="60"/>
-      <c r="K10" s="60"/>
-      <c r="L10" s="60"/>
-      <c r="M10" s="60"/>
-      <c r="N10" s="60"/>
-      <c r="O10" s="60"/>
-      <c r="P10" s="60"/>
-      <c r="Q10" s="60"/>
+      <c r="D10" s="59"/>
+      <c r="E10" s="59"/>
+      <c r="F10" s="59"/>
+      <c r="G10" s="59"/>
+      <c r="H10" s="59"/>
+      <c r="I10" s="59"/>
+      <c r="J10" s="59"/>
+      <c r="K10" s="59"/>
+      <c r="L10" s="59"/>
+      <c r="M10" s="59"/>
+      <c r="N10" s="59"/>
+      <c r="O10" s="59"/>
+      <c r="P10" s="59"/>
+      <c r="Q10" s="59"/>
     </row>
     <row r="11" spans="1:17">
-      <c r="A11" s="59"/>
-      <c r="B11" s="10" t="s">
+      <c r="A11" s="78"/>
+      <c r="B11" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="60" t="s">
+      <c r="C11" s="59" t="s">
         <v>44</v>
       </c>
-      <c r="D11" s="60"/>
-      <c r="E11" s="60"/>
-      <c r="F11" s="60"/>
-      <c r="G11" s="60"/>
-      <c r="H11" s="60"/>
-      <c r="I11" s="60"/>
-      <c r="J11" s="60"/>
-      <c r="K11" s="60"/>
-      <c r="L11" s="60"/>
-      <c r="M11" s="60"/>
-      <c r="N11" s="60"/>
-      <c r="O11" s="60"/>
-      <c r="P11" s="60"/>
-      <c r="Q11" s="60"/>
+      <c r="D11" s="59"/>
+      <c r="E11" s="59"/>
+      <c r="F11" s="59"/>
+      <c r="G11" s="59"/>
+      <c r="H11" s="59"/>
+      <c r="I11" s="59"/>
+      <c r="J11" s="59"/>
+      <c r="K11" s="59"/>
+      <c r="L11" s="59"/>
+      <c r="M11" s="59"/>
+      <c r="N11" s="59"/>
+      <c r="O11" s="59"/>
+      <c r="P11" s="59"/>
+      <c r="Q11" s="59"/>
     </row>
     <row r="12" spans="1:17">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="61" t="s">
+      <c r="B12" s="60" t="s">
         <v>44</v>
       </c>
-      <c r="C12" s="62"/>
-      <c r="D12" s="62"/>
-      <c r="E12" s="62"/>
-      <c r="F12" s="62"/>
-      <c r="G12" s="62"/>
-      <c r="H12" s="62"/>
-      <c r="I12" s="62"/>
-      <c r="J12" s="62"/>
-      <c r="K12" s="62"/>
-      <c r="L12" s="62"/>
-      <c r="M12" s="62"/>
-      <c r="N12" s="62"/>
-      <c r="O12" s="62"/>
-      <c r="P12" s="62"/>
-      <c r="Q12" s="63"/>
+      <c r="C12" s="61"/>
+      <c r="D12" s="61"/>
+      <c r="E12" s="61"/>
+      <c r="F12" s="61"/>
+      <c r="G12" s="61"/>
+      <c r="H12" s="61"/>
+      <c r="I12" s="61"/>
+      <c r="J12" s="61"/>
+      <c r="K12" s="61"/>
+      <c r="L12" s="61"/>
+      <c r="M12" s="61"/>
+      <c r="N12" s="61"/>
+      <c r="O12" s="61"/>
+      <c r="P12" s="61"/>
+      <c r="Q12" s="62"/>
     </row>
     <row r="13" spans="1:17">
-      <c r="A13" s="49" t="s">
+      <c r="A13" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="64"/>
-      <c r="C13" s="12" t="s">
+      <c r="B13" s="80"/>
+      <c r="C13" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="13"/>
-      <c r="H13" s="13"/>
-      <c r="I13" s="13"/>
-      <c r="J13" s="13"/>
-      <c r="K13" s="13"/>
-      <c r="L13" s="13"/>
-      <c r="M13" s="13"/>
-      <c r="N13" s="13"/>
-      <c r="O13" s="13"/>
-      <c r="P13" s="13"/>
-      <c r="Q13" s="14"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="12"/>
+      <c r="H13" s="12"/>
+      <c r="I13" s="12"/>
+      <c r="J13" s="12"/>
+      <c r="K13" s="12"/>
+      <c r="L13" s="12"/>
+      <c r="M13" s="12"/>
+      <c r="N13" s="12"/>
+      <c r="O13" s="12"/>
+      <c r="P13" s="12"/>
+      <c r="Q13" s="13"/>
     </row>
     <row r="14" spans="1:17">
-      <c r="A14" s="49" t="s">
+      <c r="A14" s="58" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="50"/>
-      <c r="C14" s="15" t="s">
+      <c r="B14" s="81"/>
+      <c r="C14" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
-      <c r="I14" s="7"/>
-      <c r="J14" s="7"/>
-      <c r="K14" s="7"/>
-      <c r="L14" s="7"/>
-      <c r="M14" s="7"/>
-      <c r="N14" s="7"/>
-      <c r="O14" s="7"/>
-      <c r="P14" s="7"/>
-      <c r="Q14" s="8"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="6"/>
+      <c r="I14" s="6"/>
+      <c r="J14" s="6"/>
+      <c r="K14" s="6"/>
+      <c r="L14" s="6"/>
+      <c r="M14" s="6"/>
+      <c r="N14" s="6"/>
+      <c r="O14" s="6"/>
+      <c r="P14" s="6"/>
+      <c r="Q14" s="7"/>
     </row>
     <row r="15" spans="1:17">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="75" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="67" t="s">
+      <c r="B15" s="41" t="s">
         <v>44</v>
       </c>
-      <c r="C15" s="67"/>
-      <c r="D15" s="67"/>
-      <c r="E15" s="67"/>
-      <c r="F15" s="67"/>
-      <c r="G15" s="67"/>
-      <c r="H15" s="67"/>
-      <c r="I15" s="67"/>
-      <c r="J15" s="67"/>
-      <c r="K15" s="67"/>
-      <c r="L15" s="67"/>
-      <c r="M15" s="67"/>
-      <c r="N15" s="67"/>
-      <c r="O15" s="67"/>
-      <c r="P15" s="67"/>
-      <c r="Q15" s="67"/>
+      <c r="C15" s="41"/>
+      <c r="D15" s="41"/>
+      <c r="E15" s="41"/>
+      <c r="F15" s="41"/>
+      <c r="G15" s="41"/>
+      <c r="H15" s="41"/>
+      <c r="I15" s="41"/>
+      <c r="J15" s="41"/>
+      <c r="K15" s="41"/>
+      <c r="L15" s="41"/>
+      <c r="M15" s="41"/>
+      <c r="N15" s="41"/>
+      <c r="O15" s="41"/>
+      <c r="P15" s="41"/>
+      <c r="Q15" s="41"/>
     </row>
     <row r="16" spans="1:17">
-      <c r="A16" s="73" t="s">
+      <c r="A16" s="78" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="74"/>
-      <c r="C16" s="75"/>
-      <c r="D16" s="75"/>
-      <c r="E16" s="75"/>
-      <c r="F16" s="75"/>
-      <c r="G16" s="74"/>
-      <c r="H16" s="74"/>
-      <c r="I16" s="74"/>
-      <c r="J16" s="74"/>
-      <c r="K16" s="74"/>
-      <c r="L16" s="74"/>
-      <c r="M16" s="75"/>
-      <c r="N16" s="75"/>
-      <c r="O16" s="75"/>
-      <c r="P16" s="75"/>
-      <c r="Q16" s="76"/>
+      <c r="B16" s="79"/>
+      <c r="C16" s="82"/>
+      <c r="D16" s="82"/>
+      <c r="E16" s="82"/>
+      <c r="F16" s="82"/>
+      <c r="G16" s="79"/>
+      <c r="H16" s="79"/>
+      <c r="I16" s="79"/>
+      <c r="J16" s="79"/>
+      <c r="K16" s="79"/>
+      <c r="L16" s="79"/>
+      <c r="M16" s="82"/>
+      <c r="N16" s="82"/>
+      <c r="O16" s="82"/>
+      <c r="P16" s="82"/>
+      <c r="Q16" s="83"/>
     </row>
     <row r="17" spans="1:17">
-      <c r="A17" s="65" t="s">
+      <c r="A17" s="84" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="65"/>
-      <c r="C17" s="53"/>
-      <c r="D17" s="77"/>
-      <c r="E17" s="77"/>
-      <c r="F17" s="54"/>
-      <c r="G17" s="78" t="s">
+      <c r="B17" s="84"/>
+      <c r="C17" s="47"/>
+      <c r="D17" s="48"/>
+      <c r="E17" s="48"/>
+      <c r="F17" s="49"/>
+      <c r="G17" s="92" t="s">
         <v>22</v>
       </c>
-      <c r="H17" s="79"/>
-      <c r="I17" s="79"/>
-      <c r="J17" s="79"/>
-      <c r="K17" s="79"/>
-      <c r="L17" s="80"/>
-      <c r="M17" s="81">
+      <c r="H17" s="70"/>
+      <c r="I17" s="70"/>
+      <c r="J17" s="70"/>
+      <c r="K17" s="70"/>
+      <c r="L17" s="71"/>
+      <c r="M17" s="50">
         <v>16</v>
       </c>
-      <c r="N17" s="82"/>
-      <c r="O17" s="83" t="s">
+      <c r="N17" s="51"/>
+      <c r="O17" s="52" t="s">
         <v>23</v>
       </c>
-      <c r="P17" s="83"/>
-      <c r="Q17" s="84"/>
+      <c r="P17" s="52"/>
+      <c r="Q17" s="53"/>
     </row>
     <row r="18" spans="1:17">
-      <c r="A18" s="90" t="s">
+      <c r="A18" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="B18" s="91"/>
-      <c r="C18" s="67">
+      <c r="B18" s="40"/>
+      <c r="C18" s="41">
         <v>1</v>
       </c>
-      <c r="D18" s="67"/>
-      <c r="E18" s="67"/>
-      <c r="F18" s="92"/>
-      <c r="G18" s="73" t="s">
+      <c r="D18" s="41"/>
+      <c r="E18" s="41"/>
+      <c r="F18" s="42"/>
+      <c r="G18" s="78" t="s">
         <v>25</v>
       </c>
-      <c r="H18" s="73"/>
-      <c r="I18" s="73"/>
-      <c r="J18" s="73"/>
-      <c r="K18" s="73"/>
-      <c r="L18" s="73"/>
-      <c r="M18" s="88">
+      <c r="H18" s="78"/>
+      <c r="I18" s="78"/>
+      <c r="J18" s="78"/>
+      <c r="K18" s="78"/>
+      <c r="L18" s="78"/>
+      <c r="M18" s="43">
         <v>16</v>
       </c>
-      <c r="N18" s="88"/>
-      <c r="O18" s="42" t="s">
+      <c r="N18" s="43"/>
+      <c r="O18" s="44" t="s">
         <v>23</v>
       </c>
-      <c r="P18" s="42"/>
-      <c r="Q18" s="89"/>
+      <c r="P18" s="44"/>
+      <c r="Q18" s="45"/>
     </row>
     <row r="19" spans="1:17">
-      <c r="A19" s="85" t="s">
+      <c r="A19" s="90" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="85"/>
-      <c r="C19" s="67" t="s">
+      <c r="B19" s="90"/>
+      <c r="C19" s="41" t="s">
         <v>46</v>
       </c>
-      <c r="D19" s="67"/>
-      <c r="E19" s="67"/>
-      <c r="F19" s="67"/>
-      <c r="G19" s="86" t="s">
+      <c r="D19" s="41"/>
+      <c r="E19" s="41"/>
+      <c r="F19" s="41"/>
+      <c r="G19" s="91" t="s">
         <v>27</v>
       </c>
-      <c r="H19" s="86"/>
-      <c r="I19" s="86"/>
-      <c r="J19" s="86"/>
-      <c r="K19" s="86"/>
-      <c r="L19" s="86"/>
-      <c r="M19" s="87">
+      <c r="H19" s="91"/>
+      <c r="I19" s="91"/>
+      <c r="J19" s="91"/>
+      <c r="K19" s="91"/>
+      <c r="L19" s="91"/>
+      <c r="M19" s="54">
         <f>M17-M18</f>
         <v>0</v>
       </c>
-      <c r="N19" s="88"/>
-      <c r="O19" s="42" t="s">
+      <c r="N19" s="43"/>
+      <c r="O19" s="44" t="s">
         <v>23</v>
       </c>
-      <c r="P19" s="42"/>
-      <c r="Q19" s="89"/>
+      <c r="P19" s="44"/>
+      <c r="Q19" s="45"/>
     </row>
     <row r="20" spans="1:17">
-      <c r="A20" s="65" t="s">
+      <c r="A20" s="84" t="s">
         <v>28</v>
       </c>
-      <c r="B20" s="66"/>
-      <c r="C20" s="67" t="s">
+      <c r="B20" s="85"/>
+      <c r="C20" s="41" t="s">
         <v>46</v>
       </c>
-      <c r="D20" s="67"/>
-      <c r="E20" s="67"/>
-      <c r="F20" s="67"/>
-      <c r="G20" s="67"/>
-      <c r="H20" s="67"/>
-      <c r="I20" s="67"/>
-      <c r="J20" s="67"/>
-      <c r="K20" s="67"/>
-      <c r="L20" s="67"/>
-      <c r="M20" s="67"/>
-      <c r="N20" s="67"/>
-      <c r="O20" s="67"/>
-      <c r="P20" s="67"/>
-      <c r="Q20" s="67"/>
+      <c r="D20" s="41"/>
+      <c r="E20" s="41"/>
+      <c r="F20" s="41"/>
+      <c r="G20" s="41"/>
+      <c r="H20" s="41"/>
+      <c r="I20" s="41"/>
+      <c r="J20" s="41"/>
+      <c r="K20" s="41"/>
+      <c r="L20" s="41"/>
+      <c r="M20" s="41"/>
+      <c r="N20" s="41"/>
+      <c r="O20" s="41"/>
+      <c r="P20" s="41"/>
+      <c r="Q20" s="41"/>
     </row>
     <row r="21" spans="1:17" ht="15" customHeight="1">
-      <c r="A21" s="68" t="s">
+      <c r="A21" s="86" t="s">
         <v>29</v>
       </c>
-      <c r="B21" s="69"/>
-      <c r="C21" s="72" t="s">
+      <c r="B21" s="87"/>
+      <c r="C21" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="D21" s="72"/>
-      <c r="E21" s="72"/>
-      <c r="F21" s="72"/>
-      <c r="G21" s="72"/>
-      <c r="H21" s="72"/>
-      <c r="I21" s="72"/>
-      <c r="J21" s="72"/>
-      <c r="K21" s="72"/>
-      <c r="L21" s="72"/>
-      <c r="M21" s="72"/>
-      <c r="N21" s="72"/>
-      <c r="O21" s="72"/>
-      <c r="P21" s="72"/>
-      <c r="Q21" s="72"/>
+      <c r="D21" s="46"/>
+      <c r="E21" s="46"/>
+      <c r="F21" s="46"/>
+      <c r="G21" s="46"/>
+      <c r="H21" s="46"/>
+      <c r="I21" s="46"/>
+      <c r="J21" s="46"/>
+      <c r="K21" s="46"/>
+      <c r="L21" s="46"/>
+      <c r="M21" s="46"/>
+      <c r="N21" s="46"/>
+      <c r="O21" s="46"/>
+      <c r="P21" s="46"/>
+      <c r="Q21" s="46"/>
     </row>
     <row r="22" spans="1:17" ht="14.25" customHeight="1">
-      <c r="A22" s="70"/>
-      <c r="B22" s="71"/>
-      <c r="C22" s="72"/>
-      <c r="D22" s="72"/>
-      <c r="E22" s="72"/>
-      <c r="F22" s="72"/>
-      <c r="G22" s="72"/>
-      <c r="H22" s="72"/>
-      <c r="I22" s="72"/>
-      <c r="J22" s="72"/>
-      <c r="K22" s="72"/>
-      <c r="L22" s="72"/>
-      <c r="M22" s="72"/>
-      <c r="N22" s="72"/>
-      <c r="O22" s="72"/>
-      <c r="P22" s="72"/>
-      <c r="Q22" s="72"/>
+      <c r="A22" s="88"/>
+      <c r="B22" s="89"/>
+      <c r="C22" s="46"/>
+      <c r="D22" s="46"/>
+      <c r="E22" s="46"/>
+      <c r="F22" s="46"/>
+      <c r="G22" s="46"/>
+      <c r="H22" s="46"/>
+      <c r="I22" s="46"/>
+      <c r="J22" s="46"/>
+      <c r="K22" s="46"/>
+      <c r="L22" s="46"/>
+      <c r="M22" s="46"/>
+      <c r="N22" s="46"/>
+      <c r="O22" s="46"/>
+      <c r="P22" s="46"/>
+      <c r="Q22" s="46"/>
     </row>
     <row r="24" spans="1:17" ht="31.5" customHeight="1">
-      <c r="A24" s="41" t="s">
+      <c r="A24" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="41"/>
-      <c r="C24" s="41"/>
-      <c r="D24" s="41"/>
-      <c r="E24" s="41"/>
-      <c r="F24" s="41"/>
-      <c r="G24" s="41"/>
-      <c r="H24" s="41"/>
-      <c r="I24" s="41"/>
-      <c r="J24" s="41"/>
-      <c r="K24" s="41"/>
-      <c r="L24" s="41"/>
-      <c r="M24" s="41"/>
-      <c r="N24" s="41"/>
-      <c r="O24" s="41"/>
-      <c r="P24" s="41"/>
-      <c r="Q24" s="41"/>
+      <c r="B24" s="35"/>
+      <c r="C24" s="35"/>
+      <c r="D24" s="35"/>
+      <c r="E24" s="35"/>
+      <c r="F24" s="35"/>
+      <c r="G24" s="35"/>
+      <c r="H24" s="35"/>
+      <c r="I24" s="35"/>
+      <c r="J24" s="35"/>
+      <c r="K24" s="35"/>
+      <c r="L24" s="35"/>
+      <c r="M24" s="35"/>
+      <c r="N24" s="35"/>
+      <c r="O24" s="35"/>
+      <c r="P24" s="35"/>
+      <c r="Q24" s="35"/>
     </row>
     <row r="26" spans="1:17">
-      <c r="A26" s="96" t="s">
+      <c r="A26" s="38" t="s">
         <v>33</v>
       </c>
-      <c r="B26" s="96"/>
-      <c r="C26" s="96"/>
-      <c r="F26" s="96" t="s">
+      <c r="B26" s="38"/>
+      <c r="C26" s="38"/>
+      <c r="F26" s="38" t="s">
         <v>31</v>
       </c>
-      <c r="G26" s="96"/>
-      <c r="H26" s="96"/>
-      <c r="I26" s="96"/>
-      <c r="J26" s="96"/>
-      <c r="K26" s="96"/>
-      <c r="L26" s="96"/>
-      <c r="M26" s="96"/>
-      <c r="N26" s="96"/>
-      <c r="O26" s="96"/>
-      <c r="P26" s="96"/>
-      <c r="Q26" s="96"/>
+      <c r="G26" s="38"/>
+      <c r="H26" s="38"/>
+      <c r="I26" s="38"/>
+      <c r="J26" s="38"/>
+      <c r="K26" s="38"/>
+      <c r="L26" s="38"/>
+      <c r="M26" s="38"/>
+      <c r="N26" s="38"/>
+      <c r="O26" s="38"/>
+      <c r="P26" s="38"/>
+      <c r="Q26" s="38"/>
     </row>
     <row r="27" spans="1:17" ht="57.75" customHeight="1">
-      <c r="A27" s="94"/>
-      <c r="B27" s="94"/>
-      <c r="C27" s="94"/>
-      <c r="F27" s="94"/>
-      <c r="G27" s="94"/>
-      <c r="H27" s="94"/>
-      <c r="I27" s="94"/>
-      <c r="J27" s="94"/>
-      <c r="K27" s="94"/>
-      <c r="L27" s="94"/>
-      <c r="M27" s="94"/>
-      <c r="N27" s="94"/>
-      <c r="O27" s="94"/>
-      <c r="P27" s="94"/>
-      <c r="Q27" s="94"/>
-    </row>
-    <row r="28" spans="1:17" s="16" customFormat="1">
-      <c r="A28" s="95" t="s">
+      <c r="A27" s="36"/>
+      <c r="B27" s="36"/>
+      <c r="C27" s="36"/>
+      <c r="F27" s="36"/>
+      <c r="G27" s="36"/>
+      <c r="H27" s="36"/>
+      <c r="I27" s="36"/>
+      <c r="J27" s="36"/>
+      <c r="K27" s="36"/>
+      <c r="L27" s="36"/>
+      <c r="M27" s="36"/>
+      <c r="N27" s="36"/>
+      <c r="O27" s="36"/>
+      <c r="P27" s="36"/>
+      <c r="Q27" s="36"/>
+    </row>
+    <row r="28" spans="1:17" s="15" customFormat="1">
+      <c r="A28" s="37" t="s">
         <v>57</v>
       </c>
-      <c r="B28" s="95"/>
-      <c r="C28" s="95"/>
-      <c r="F28" s="95"/>
-      <c r="G28" s="95"/>
-      <c r="H28" s="95"/>
-      <c r="I28" s="95"/>
-      <c r="J28" s="95"/>
-      <c r="K28" s="95"/>
-      <c r="L28" s="95"/>
-      <c r="M28" s="95"/>
-      <c r="N28" s="95"/>
-      <c r="O28" s="95"/>
-      <c r="P28" s="95"/>
-      <c r="Q28" s="95"/>
-    </row>
-    <row r="33" spans="1:17" ht="59" customHeight="1"/>
+      <c r="B28" s="37"/>
+      <c r="C28" s="37"/>
+      <c r="F28" s="37"/>
+      <c r="G28" s="37"/>
+      <c r="H28" s="37"/>
+      <c r="I28" s="37"/>
+      <c r="J28" s="37"/>
+      <c r="K28" s="37"/>
+      <c r="L28" s="37"/>
+      <c r="M28" s="37"/>
+      <c r="N28" s="37"/>
+      <c r="O28" s="37"/>
+      <c r="P28" s="37"/>
+      <c r="Q28" s="37"/>
+    </row>
+    <row r="33" spans="1:17" ht="16" customHeight="1">
+      <c r="D33" s="76"/>
+    </row>
     <row r="34" spans="1:17" ht="32" customHeight="1">
-      <c r="A34" s="93" t="s">
+      <c r="A34" s="34" t="s">
         <v>32</v>
       </c>
-      <c r="B34" s="93"/>
-      <c r="C34" s="93"/>
-      <c r="D34" s="93"/>
-      <c r="E34" s="93"/>
-      <c r="F34" s="93"/>
-      <c r="G34" s="93"/>
-      <c r="H34" s="93"/>
-      <c r="I34" s="93"/>
-      <c r="J34" s="93"/>
-      <c r="K34" s="93"/>
-      <c r="L34" s="93"/>
-      <c r="M34" s="93"/>
-      <c r="N34" s="93"/>
-      <c r="O34" s="93"/>
-      <c r="P34" s="93"/>
-      <c r="Q34" s="93"/>
+      <c r="B34" s="34"/>
+      <c r="C34" s="34"/>
+      <c r="D34" s="34"/>
+      <c r="E34" s="34"/>
+      <c r="F34" s="34"/>
+      <c r="G34" s="34"/>
+      <c r="H34" s="34"/>
+      <c r="I34" s="34"/>
+      <c r="J34" s="34"/>
+      <c r="K34" s="34"/>
+      <c r="L34" s="34"/>
+      <c r="M34" s="34"/>
+      <c r="N34" s="34"/>
+      <c r="O34" s="34"/>
+      <c r="P34" s="34"/>
+      <c r="Q34" s="34"/>
     </row>
     <row r="35" spans="1:17" ht="14.5" customHeight="1"/>
     <row r="36" spans="1:17" ht="16.5" customHeight="1"/>
     <row r="37" spans="1:17" ht="39.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="49">
-    <mergeCell ref="A34:Q34"/>
-    <mergeCell ref="A24:Q24"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="F27:Q27"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="F28:Q28"/>
-    <mergeCell ref="A26:C26"/>
-    <mergeCell ref="F26:Q26"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="C18:F18"/>
-    <mergeCell ref="G18:L18"/>
-    <mergeCell ref="M18:N18"/>
-    <mergeCell ref="O18:Q18"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="E6:J6"/>
+    <mergeCell ref="K6:Q6"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A3:Q3"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="E5:J5"/>
+    <mergeCell ref="K5:Q5"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="O7:P7"/>
+    <mergeCell ref="B8:Q8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C9:Q9"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="C10:Q10"/>
+    <mergeCell ref="C11:Q11"/>
+    <mergeCell ref="B12:Q12"/>
+    <mergeCell ref="A13:B13"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="C20:Q20"/>
     <mergeCell ref="A21:B22"/>
@@ -2216,26 +2221,19 @@
     <mergeCell ref="G19:L19"/>
     <mergeCell ref="M19:N19"/>
     <mergeCell ref="O19:Q19"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="K7:L7"/>
-    <mergeCell ref="M7:N7"/>
-    <mergeCell ref="O7:P7"/>
-    <mergeCell ref="B8:Q8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C9:Q9"/>
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="C10:Q10"/>
-    <mergeCell ref="C11:Q11"/>
-    <mergeCell ref="B12:Q12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="E6:J6"/>
-    <mergeCell ref="K6:Q6"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="E5:J5"/>
-    <mergeCell ref="K5:Q5"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="C18:F18"/>
+    <mergeCell ref="G18:L18"/>
+    <mergeCell ref="M18:N18"/>
+    <mergeCell ref="O18:Q18"/>
+    <mergeCell ref="A34:Q34"/>
+    <mergeCell ref="A24:Q24"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="F27:Q27"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="F28:Q28"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="F26:Q26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.80208333333333337" top="1.5625" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>